<commit_message>
Producto 2 con capturas de todas las alas y del final
</commit_message>
<xml_diff>
--- a/Documentacion/Producto2/PérezAlcántaraAlejandro_producción_10D_Sprint2.xlsx
+++ b/Documentacion/Producto2/PérezAlcántaraAlejandro_producción_10D_Sprint2.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="412">
   <si>
     <t xml:space="preserve">FEATURE LOG - ECOS DEL GRIMORIO (actualizado al Sprint 2)</t>
   </si>
@@ -503,6 +503,12 @@
     <t xml:space="preserve">Sprint Review del Sprint 2</t>
   </si>
   <si>
+    <t xml:space="preserve">T36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corregir el acertijo de la caja del Ala de Viento (B-014)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total horas:</t>
   </si>
   <si>
@@ -572,7 +578,7 @@
     <t xml:space="preserve">Corregir el final de Elenora, agregar capturas y compilación del .exe, actualizar producción.</t>
   </si>
   <si>
-    <t xml:space="preserve">El final no terminaba al vencer a Elenora (B-012); el panel de depuración se abría con L3 + R3 (B-013).</t>
+    <t xml:space="preserve">El final no terminaba al vencer a Elenora (B-012); el panel de depuración se abría con L3 + R3 (B-013); no se abría el pasadizo del Ala de Viento (B-014).</t>
   </si>
   <si>
     <t xml:space="preserve">PROJECT CHART - Estado general del proyecto</t>
@@ -761,18 +767,27 @@
     <t xml:space="preserve">La secuencia final dependía de que todos los eventos terminaran sin error; ahora hay un respaldo que termina el juego siempre.</t>
   </si>
   <si>
+    <t xml:space="preserve">B-013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se abría un panel de estadísticas de Unity al apretar los dos sticks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rendering Debugger de URP activo en tiempo de juego (L3 + R3); se desactiva en CapturaPantalla.cs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No se podía abrir el pasadizo de la Página Perdida del Ala de Viento.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La caja estaba casi en la orilla del suelo y podía caer al vacío; las puertas rúnicas no explicaban cómo abrirse. Se dio más espacio, la caja regresa a su lugar si se cae y las puertas dan una pista.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Por verificar</t>
   </si>
   <si>
-    <t xml:space="preserve">B-013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Se abría un panel de estadísticas de Unity al apretar los dos sticks.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rendering Debugger de URP activo en tiempo de juego (L3 + R3); se desactiva en CapturaPantalla.cs.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Corregidos:</t>
   </si>
   <si>
@@ -953,6 +968,9 @@
     <t xml:space="preserve">Lira cae lento; la caja abre la puerta rúnica.</t>
   </si>
   <si>
+    <t xml:space="preserve">No se podía abrir (B-014). Corregido, falta probar.</t>
+  </si>
+  <si>
     <t xml:space="preserve">PA-12</t>
   </si>
   <si>
@@ -965,7 +983,7 @@
     <t xml:space="preserve">¡VICTORIA!, epílogo y créditos; al final regresa al menú.</t>
   </si>
   <si>
-    <t xml:space="preserve">No terminaba (B-012). Corregido, falta probar.</t>
+    <t xml:space="preserve">No terminaba (B-012). Corregido: sale ¡VICTORIA!, epílogo y créditos.</t>
   </si>
   <si>
     <t xml:space="preserve">PA-13</t>
@@ -2057,31 +2075,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>164</c:v>
+                  <c:v>165</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>148</c:v>
+                  <c:v>148.9</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>136</c:v>
+                  <c:v>136.8</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>120</c:v>
+                  <c:v>120.7</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>104</c:v>
+                  <c:v>104.6</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>100</c:v>
+                  <c:v>100.6</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>92</c:v>
+                  <c:v>92.6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>64</c:v>
+                  <c:v>64.4</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>36</c:v>
+                  <c:v>36.2</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>8</c:v>
@@ -2195,22 +2213,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>164</c:v>
+                  <c:v>165</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>164</c:v>
+                  <c:v>165</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>164</c:v>
+                  <c:v>165</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>126</c:v>
+                  <c:v>127</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>73</c:v>
+                  <c:v>74</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>23</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>15</c:v>
@@ -2228,11 +2246,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="94603327"/>
-        <c:axId val="30785891"/>
+        <c:axId val="96940786"/>
+        <c:axId val="53340935"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="94603327"/>
+        <c:axId val="96940786"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2298,7 +2316,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30785891"/>
+        <c:crossAx val="53340935"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2306,7 +2324,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="30785891"/>
+        <c:axId val="53340935"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2382,7 +2400,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94603327"/>
+        <c:crossAx val="96940786"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2567,22 +2585,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>35</c:v>
+                  <c:v>36</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>35</c:v>
+                  <c:v>36</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>35</c:v>
+                  <c:v>36</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>28</c:v>
+                  <c:v>29</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>19</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>7</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>4</c:v>
@@ -2699,7 +2717,7 @@
                   <c:v>28</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>31</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2714,11 +2732,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="46734740"/>
-        <c:axId val="5460073"/>
+        <c:axId val="2262243"/>
+        <c:axId val="47176895"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="46734740"/>
+        <c:axId val="2262243"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2784,7 +2802,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5460073"/>
+        <c:crossAx val="47176895"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2792,7 +2810,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="5460073"/>
+        <c:axId val="47176895"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2868,7 +2886,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46734740"/>
+        <c:crossAx val="2262243"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3840,7 +3858,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3849,7 +3867,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3858,16 +3876,16 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>4</v>
@@ -3875,13 +3893,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>139</v>
@@ -3893,13 +3911,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>91</v>
@@ -3911,13 +3929,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>117</v>
@@ -3929,13 +3947,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>99</v>
@@ -3947,16 +3965,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="E8" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C8,FIND(",",C8&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -3965,13 +3983,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>135</v>
@@ -3983,16 +4001,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="E10" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C10,FIND(",",C10&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4001,16 +4019,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="E11" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C11,FIND(",",C11&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4019,13 +4037,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>125</v>
@@ -4037,16 +4055,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="E13" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C13,FIND(",",C13&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4055,16 +4073,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="E14" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C14,FIND(",",C14&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4073,13 +4091,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>133</v>
@@ -4091,16 +4109,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="E16" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C16,FIND(",",C16&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4109,16 +4127,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="E17" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C17,FIND(",",C17&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4127,13 +4145,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>111</v>
@@ -4145,13 +4163,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>127</v>
@@ -4163,16 +4181,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="E20" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C20,FIND(",",C20&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4181,16 +4199,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="E21" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C21,FIND(",",C21&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4199,16 +4217,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="E22" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C22,FIND(",",C22&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4270,39 +4288,39 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="B4" s="5" t="str">
-        <f aca="false">COUNTIF('Sprint Backlog'!$F$4:$F$38,"Terminado")&amp;" de "&amp;COUNTA('Sprint Backlog'!$A$4:$A$38)</f>
-        <v>31 de 35</v>
+        <f aca="false">COUNTIF('Sprint Backlog'!$F$4:$F$39,"Terminado")&amp;" de "&amp;COUNTA('Sprint Backlog'!$A$4:$A$39)</f>
+        <v>32 de 36</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="B5" s="5" t="str">
-        <f aca="false">SUMIF('Sprint Backlog'!$F$4:$F$38,"Terminado",'Sprint Backlog'!$G$4:$G$38)&amp;" de "&amp;'Sprint Backlog'!$G$40&amp;" hrs"</f>
-        <v>149 de 164 hrs</v>
+        <f aca="false">SUMIF('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$G$4:$G$39)&amp;" de "&amp;'Sprint Backlog'!$G$41&amp;" hrs"</f>
+        <v>150 de 165 hrs</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="B6" s="5" t="str">
         <f aca="false">COUNTIF('Feature Log'!$C$4:$C$29,"Terminado")&amp;" de "&amp;COUNTA('Feature Log'!$A$4:$A$29)</f>
@@ -4311,60 +4329,60 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="B7" s="5" t="str">
-        <f aca="false">COUNTIF(Buglist!$E$4:$E$16,"Corregido")&amp;" de "&amp;COUNTA(Buglist!$A$4:$A$16)</f>
-        <v>12 de 13</v>
+        <f aca="false">COUNTIF(Buglist!$E$4:$E$17,"Corregido")&amp;" de "&amp;COUNTA(Buglist!$A$4:$A$17)</f>
+        <v>13 de 14</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="B8" s="5" t="str">
         <f aca="false">COUNTIF('Pruebas Alfa'!$G$4:$G$17,"Aprobada")&amp;" de "&amp;COUNTA('Pruebas Alfa'!$A$4:$A$17)</f>
-        <v>8 de 14</v>
+        <v>9 de 14</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
     </row>
   </sheetData>
@@ -4585,7 +4603,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -5656,31 +5674,60 @@
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F40" s="8" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="G40" s="8" t="n">
-        <f aca="false">SUM(G4:G38)</f>
-        <v>164</v>
+      <c r="B39" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" s="6" t="n">
+        <v>46302</v>
+      </c>
+      <c r="I39" s="6" t="n">
+        <v>46302</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F41" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="G41" s="8" t="str">
-        <f aca="false">COUNTIF(F4:F38,"Terminado")&amp;" de "&amp;COUNTA(A4:A38)</f>
-        <v>31 de 35</v>
+        <v>159</v>
+      </c>
+      <c r="G41" s="8" t="n">
+        <f aca="false">SUM(G4:G39)</f>
+        <v>165</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F42" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="G42" s="9" t="n">
-        <f aca="false">SUMIF(F4:F38,"Terminado",G4:G38)/G40</f>
-        <v>0.908536585365854</v>
+        <v>160</v>
+      </c>
+      <c r="G42" s="8" t="str">
+        <f aca="false">COUNTIF(F4:F39,"Terminado")&amp;" de "&amp;COUNTA(A4:A39)</f>
+        <v>32 de 36</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F43" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="G43" s="9" t="n">
+        <f aca="false">SUMIF(F4:F39,"Terminado",G4:G39)/G41</f>
+        <v>0.909090909090909</v>
       </c>
     </row>
   </sheetData>
@@ -5688,7 +5735,7 @@
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F4:F38">
+  <conditionalFormatting sqref="F4:F39">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminado"</formula>
     </cfRule>
@@ -5715,7 +5762,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F4:F38" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F4:F39" type="list">
       <formula1>"Terminado,En desarrollo,Planeado"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5744,7 +5791,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5752,7 +5799,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5760,16 +5807,16 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5777,13 +5824,13 @@
         <v>46284</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5791,13 +5838,13 @@
         <v>46295</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5805,13 +5852,13 @@
         <v>46299</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5819,27 +5866,27 @@
         <v>46300</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="n">
         <v>46302</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -5872,14 +5919,14 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5887,10 +5934,10 @@
         <v>4</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5934,7 +5981,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B7" s="13" t="n">
         <f aca="false">COUNTIF('Feature Log'!$C$4:$C$29,A7)</f>
@@ -5947,7 +5994,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B8" s="15" t="n">
         <f aca="false">SUM(B4:B7)</f>
@@ -5985,7 +6032,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5993,7 +6040,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6003,16 +6050,16 @@
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6020,16 +6067,16 @@
         <v>46284</v>
       </c>
       <c r="B4" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$40*('Sprint Plan'!$D$5-A4)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>164</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A4)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>165</v>
       </c>
       <c r="C4" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$40-SUMIFS('Sprint Backlog'!$G$4:$G$38,'Sprint Backlog'!$F$4:$F$38,"Terminado",'Sprint Backlog'!$I$4:$I$38,"&lt;="&amp;A4)</f>
-        <v>164</v>
+        <f aca="false">'Sprint Backlog'!$G$41-SUMIFS('Sprint Backlog'!$G$4:$G$39,'Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A4)</f>
+        <v>165</v>
       </c>
       <c r="D4" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$38)-COUNTIFS('Sprint Backlog'!$F$4:$F$38,"Terminado",'Sprint Backlog'!$I$4:$I$38,"&lt;="&amp;A4)</f>
-        <v>35</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-COUNTIFS('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A4)</f>
+        <v>36</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6037,16 +6084,16 @@
         <v>46288</v>
       </c>
       <c r="B5" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$40*('Sprint Plan'!$D$5-A5)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>148</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A5)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>148.9</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$40-SUMIFS('Sprint Backlog'!$G$4:$G$38,'Sprint Backlog'!$F$4:$F$38,"Terminado",'Sprint Backlog'!$I$4:$I$38,"&lt;="&amp;A5)</f>
-        <v>164</v>
+        <f aca="false">'Sprint Backlog'!$G$41-SUMIFS('Sprint Backlog'!$G$4:$G$39,'Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A5)</f>
+        <v>165</v>
       </c>
       <c r="D5" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$38)-COUNTIFS('Sprint Backlog'!$F$4:$F$38,"Terminado",'Sprint Backlog'!$I$4:$I$38,"&lt;="&amp;A5)</f>
-        <v>35</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-COUNTIFS('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A5)</f>
+        <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6054,16 +6101,16 @@
         <v>46291</v>
       </c>
       <c r="B6" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$40*('Sprint Plan'!$D$5-A6)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>136</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A6)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>136.8</v>
       </c>
       <c r="C6" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$40-SUMIFS('Sprint Backlog'!$G$4:$G$38,'Sprint Backlog'!$F$4:$F$38,"Terminado",'Sprint Backlog'!$I$4:$I$38,"&lt;="&amp;A6)</f>
-        <v>164</v>
+        <f aca="false">'Sprint Backlog'!$G$41-SUMIFS('Sprint Backlog'!$G$4:$G$39,'Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A6)</f>
+        <v>165</v>
       </c>
       <c r="D6" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$38)-COUNTIFS('Sprint Backlog'!$F$4:$F$38,"Terminado",'Sprint Backlog'!$I$4:$I$38,"&lt;="&amp;A6)</f>
-        <v>35</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-COUNTIFS('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A6)</f>
+        <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6071,16 +6118,16 @@
         <v>46295</v>
       </c>
       <c r="B7" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$40*('Sprint Plan'!$D$5-A7)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>120</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A7)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>120.7</v>
       </c>
       <c r="C7" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$40-SUMIFS('Sprint Backlog'!$G$4:$G$38,'Sprint Backlog'!$F$4:$F$38,"Terminado",'Sprint Backlog'!$I$4:$I$38,"&lt;="&amp;A7)</f>
-        <v>126</v>
+        <f aca="false">'Sprint Backlog'!$G$41-SUMIFS('Sprint Backlog'!$G$4:$G$39,'Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A7)</f>
+        <v>127</v>
       </c>
       <c r="D7" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$38)-COUNTIFS('Sprint Backlog'!$F$4:$F$38,"Terminado",'Sprint Backlog'!$I$4:$I$38,"&lt;="&amp;A7)</f>
-        <v>28</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-COUNTIFS('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A7)</f>
+        <v>29</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6088,16 +6135,16 @@
         <v>46299</v>
       </c>
       <c r="B8" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$40*('Sprint Plan'!$D$5-A8)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>104</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A8)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>104.6</v>
       </c>
       <c r="C8" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$40-SUMIFS('Sprint Backlog'!$G$4:$G$38,'Sprint Backlog'!$F$4:$F$38,"Terminado",'Sprint Backlog'!$I$4:$I$38,"&lt;="&amp;A8)</f>
-        <v>73</v>
+        <f aca="false">'Sprint Backlog'!$G$41-SUMIFS('Sprint Backlog'!$G$4:$G$39,'Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A8)</f>
+        <v>74</v>
       </c>
       <c r="D8" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$38)-COUNTIFS('Sprint Backlog'!$F$4:$F$38,"Terminado",'Sprint Backlog'!$I$4:$I$38,"&lt;="&amp;A8)</f>
-        <v>19</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-COUNTIFS('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A8)</f>
+        <v>20</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6105,16 +6152,16 @@
         <v>46300</v>
       </c>
       <c r="B9" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$40*('Sprint Plan'!$D$5-A9)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>100</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A9)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>100.6</v>
       </c>
       <c r="C9" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$40-SUMIFS('Sprint Backlog'!$G$4:$G$38,'Sprint Backlog'!$F$4:$F$38,"Terminado",'Sprint Backlog'!$I$4:$I$38,"&lt;="&amp;A9)</f>
-        <v>23</v>
+        <f aca="false">'Sprint Backlog'!$G$41-SUMIFS('Sprint Backlog'!$G$4:$G$39,'Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A9)</f>
+        <v>24</v>
       </c>
       <c r="D9" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$38)-COUNTIFS('Sprint Backlog'!$F$4:$F$38,"Terminado",'Sprint Backlog'!$I$4:$I$38,"&lt;="&amp;A9)</f>
-        <v>7</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-COUNTIFS('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A9)</f>
+        <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6122,15 +6169,15 @@
         <v>46302</v>
       </c>
       <c r="B10" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$40*('Sprint Plan'!$D$5-A10)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>92</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A10)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>92.6</v>
       </c>
       <c r="C10" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$40-SUMIFS('Sprint Backlog'!$G$4:$G$38,'Sprint Backlog'!$F$4:$F$38,"Terminado",'Sprint Backlog'!$I$4:$I$38,"&lt;="&amp;A10)</f>
+        <f aca="false">'Sprint Backlog'!$G$41-SUMIFS('Sprint Backlog'!$G$4:$G$39,'Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A10)</f>
         <v>15</v>
       </c>
       <c r="D10" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$38)-COUNTIFS('Sprint Backlog'!$F$4:$F$38,"Terminado",'Sprint Backlog'!$I$4:$I$38,"&lt;="&amp;A10)</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-COUNTIFS('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A10)</f>
         <v>4</v>
       </c>
     </row>
@@ -6139,8 +6186,8 @@
         <v>46309</v>
       </c>
       <c r="B11" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$40*('Sprint Plan'!$D$5-A11)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>64</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A11)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>64.4</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
@@ -6150,8 +6197,8 @@
         <v>46316</v>
       </c>
       <c r="B12" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$40*('Sprint Plan'!$D$5-A12)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>36</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A12)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>36.2</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
@@ -6161,7 +6208,7 @@
         <v>46323</v>
       </c>
       <c r="B13" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$40*('Sprint Plan'!$D$5-A13)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A13)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
         <v>8</v>
       </c>
       <c r="C13" s="13"/>
@@ -6172,7 +6219,7 @@
         <v>46325</v>
       </c>
       <c r="B14" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$40*('Sprint Plan'!$D$5-A14)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A14)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
         <v>0</v>
       </c>
       <c r="C14" s="13"/>
@@ -6209,25 +6256,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6237,10 +6284,10 @@
       </c>
       <c r="B4" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D4</f>
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C4" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$38)-B4</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-B4</f>
         <v>0</v>
       </c>
     </row>
@@ -6251,10 +6298,10 @@
       </c>
       <c r="B5" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D5</f>
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$38)-B5</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-B5</f>
         <v>0</v>
       </c>
     </row>
@@ -6265,10 +6312,10 @@
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D6</f>
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C6" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$38)-B6</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-B6</f>
         <v>0</v>
       </c>
     </row>
@@ -6279,10 +6326,10 @@
       </c>
       <c r="B7" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D7</f>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C7" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$38)-B7</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-B7</f>
         <v>7</v>
       </c>
     </row>
@@ -6293,10 +6340,10 @@
       </c>
       <c r="B8" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D8</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$38)-B8</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-B8</f>
         <v>16</v>
       </c>
     </row>
@@ -6307,10 +6354,10 @@
       </c>
       <c r="B9" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D9</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C9" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$38)-B9</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-B9</f>
         <v>28</v>
       </c>
     </row>
@@ -6324,8 +6371,8 @@
         <v>4</v>
       </c>
       <c r="C10" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$38)-B10</f>
-        <v>31</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-B10</f>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -6348,7 +6395,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -6363,7 +6410,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6375,7 +6422,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6387,16 +6434,16 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>4</v>
@@ -6405,27 +6452,27 @@
         <v>2</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>15</v>
@@ -6434,24 +6481,24 @@
         <v>46299</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>14</v>
@@ -6460,24 +6507,24 @@
         <v>46300</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>19</v>
@@ -6486,24 +6533,24 @@
         <v>46300</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>15</v>
@@ -6512,24 +6559,24 @@
         <v>46300</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>17</v>
@@ -6538,24 +6585,24 @@
         <v>46300</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>11</v>
@@ -6564,24 +6611,24 @@
         <v>46300</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>18</v>
@@ -6590,24 +6637,24 @@
         <v>46300</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>13</v>
@@ -6616,24 +6663,24 @@
         <v>46300</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>19</v>
@@ -6642,24 +6689,24 @@
         <v>46300</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F13" s="4" t="n">
         <v>22</v>
@@ -6668,24 +6715,24 @@
         <v>46300</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>17</v>
@@ -6694,24 +6741,24 @@
         <v>46300</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>243</v>
+        <v>208</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>11</v>
@@ -6720,24 +6767,24 @@
         <v>46302</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F16" s="4" t="n">
         <v>20</v>
@@ -6746,16 +6793,42 @@
         <v>46302</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D18" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="E18" s="8" t="str">
-        <f aca="false">COUNTIF(E4:E16,"Corregido")&amp;" de "&amp;COUNTA(A4:A16)</f>
-        <v>12 de 13</v>
+        <v>213</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D19" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="E19" s="8" t="str">
+        <f aca="false">COUNTIF(E4:E17,"Corregido")&amp;" de "&amp;COUNTA(A4:A17)</f>
+        <v>13 de 14</v>
       </c>
     </row>
   </sheetData>
@@ -6763,7 +6836,7 @@
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E4:E16">
+  <conditionalFormatting sqref="E4:E17">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminado"</formula>
     </cfRule>
@@ -6818,7 +6891,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6829,7 +6902,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6840,22 +6913,22 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>4</v>
@@ -6863,323 +6936,325 @@
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="F5" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>265</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="F6" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>265</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>20</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="F7" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="G7" s="4" t="s">
         <v>265</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>19</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>17</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>13</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>16</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="F12" s="5"/>
       <c r="G12" s="4" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="4" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="B14" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>306</v>
-      </c>
-      <c r="F14" s="5"/>
+        <v>311</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>312</v>
+      </c>
       <c r="G14" s="4" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>11</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>298</v>
+        <v>265</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>23</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="F16" s="5"/>
       <c r="G16" s="4" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>24</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="F17" s="5"/>
       <c r="G17" s="4" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F19" s="8" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="G19" s="8" t="str">
         <f aca="false">COUNTIF(G4:G17,"Aprobada")&amp;" de "&amp;COUNTA(A4:A17)</f>
-        <v>8 de 14</v>
+        <v>9 de 14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Producción del Sprint 2 al 13 de octubre: Lira pegada al suelo, controles y .exe
</commit_message>
<xml_diff>
--- a/Documentacion/Producto2/PérezAlcántaraAlejandro_producción_10D_Sprint2.xlsx
+++ b/Documentacion/Producto2/PérezAlcántaraAlejandro_producción_10D_Sprint2.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="430">
   <si>
     <t xml:space="preserve">FEATURE LOG - ECOS DEL GRIMORIO (actualizado al Sprint 2)</t>
   </si>
@@ -509,6 +509,24 @@
     <t xml:space="preserve">Corregir el acertijo de la caja del Ala de Viento (B-014)</t>
   </si>
   <si>
+    <t xml:space="preserve">T37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corregir a Lira flotando sobre el suelo (B-015)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Controles de teclado para laptop (J K L, W para apuntar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manual del jugador en PDF</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total horas:</t>
   </si>
   <si>
@@ -581,6 +599,15 @@
     <t xml:space="preserve">El final no terminaba al vencer a Elenora (B-012); el panel de depuración se abría con L3 + R3 (B-013); no se abría el pasadizo del Ala de Viento (B-014).</t>
   </si>
   <si>
+    <t xml:space="preserve">Producto 2 completo y probado el final del juego.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corregir a Lira flotando, controles de teclado para laptop, manual del jugador y generar el .exe.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El profesor notó que Lira flota sobre el suelo (B-015).</t>
+  </si>
+  <si>
     <t xml:space="preserve">PROJECT CHART - Estado general del proyecto</t>
   </si>
   <si>
@@ -788,6 +815,15 @@
     <t xml:space="preserve">Por verificar</t>
   </si>
   <si>
+    <t xml:space="preserve">B-015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El profesor notó que Lira a veces flota sobre el suelo y las plataformas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La imagen de Lira tiene 17% de espacio transparente bajo los pies y el collider se calculaba con la imagen completa. Ahora EditorHelpers.MargenesTransparentes() lee el PNG y ajusta el collider y el GroundCheck a los pies reales.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Corregidos:</t>
   </si>
   <si>
@@ -1010,6 +1046,24 @@
     <t xml:space="preserve">El juego abre en pantalla completa y se puede jugar de inicio a fin.</t>
   </si>
   <si>
+    <t xml:space="preserve">Compila sin errores (150 MB). Falta probarlo en otra computadora.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PA-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lira pisa el suelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caminar y detenerse sobre el suelo y las plataformas de cada ala.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Los pies de Lira tocan la superficie, sin espacio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flotaba (B-015). Corregido.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Aprobadas:</t>
   </si>
   <si>
@@ -1214,7 +1268,7 @@
     <t xml:space="preserve">T30, T33</t>
   </si>
   <si>
-    <t xml:space="preserve">SPRINT REVIEW - SPRINT 2 (avance al 7 de octubre de 2026)</t>
+    <t xml:space="preserve">SPRINT REVIEW - SPRINT 2 (avance al 13 de octubre de 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Meta del sprint</t>
@@ -2054,7 +2108,7 @@
                   <c:v>07/10</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>14/10</c:v>
+                  <c:v>13/10</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>21/10</c:v>
@@ -2075,34 +2129,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>165</c:v>
+                  <c:v>172</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>148.9</c:v>
+                  <c:v>155.2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>136.8</c:v>
+                  <c:v>142.6</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>120.7</c:v>
+                  <c:v>125.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>104.6</c:v>
+                  <c:v>109.1</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>100.6</c:v>
+                  <c:v>104.9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>92.6</c:v>
+                  <c:v>96.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>64.4</c:v>
+                  <c:v>71.3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>36.2</c:v>
+                  <c:v>37.8</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>8</c:v>
+                  <c:v>8.4</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
@@ -2192,7 +2246,7 @@
                   <c:v>07/10</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>14/10</c:v>
+                  <c:v>13/10</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>21/10</c:v>
@@ -2213,24 +2267,27 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>165</c:v>
+                  <c:v>172</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>165</c:v>
+                  <c:v>172</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>165</c:v>
+                  <c:v>172</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>127</c:v>
+                  <c:v>134</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>74</c:v>
+                  <c:v>81</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>24</c:v>
+                  <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="6">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>15</c:v>
                 </c:pt>
               </c:numCache>
@@ -2246,11 +2303,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="96940786"/>
-        <c:axId val="53340935"/>
+        <c:axId val="6751934"/>
+        <c:axId val="62335594"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="96940786"/>
+        <c:axId val="6751934"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2316,7 +2373,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53340935"/>
+        <c:crossAx val="62335594"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2324,7 +2381,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="53340935"/>
+        <c:axId val="62335594"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2400,7 +2457,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96940786"/>
+        <c:crossAx val="6751934"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2551,9 +2608,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Task Chart'!$A$4:$A$10</c:f>
+              <c:f>'Task Chart'!$A$4:$A$11</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>19/09</c:v>
                 </c:pt>
@@ -2574,35 +2631,41 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>07/10</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>13/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Task Chart'!$B$4:$B$10</c:f>
+              <c:f>'Task Chart'!$B$4:$B$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>36</c:v>
+                  <c:v>39</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>36</c:v>
+                  <c:v>39</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>36</c:v>
+                  <c:v>39</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>29</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>20</c:v>
+                  <c:v>23</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>4</c:v>
                 </c:pt>
               </c:numCache>
@@ -2665,9 +2728,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Task Chart'!$A$4:$A$10</c:f>
+              <c:f>'Task Chart'!$A$4:$A$11</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>19/09</c:v>
                 </c:pt>
@@ -2688,16 +2751,19 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>07/10</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>13/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Task Chart'!$C$4:$C$10</c:f>
+              <c:f>'Task Chart'!$C$4:$C$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -2718,6 +2784,9 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>35</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2732,11 +2801,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="2262243"/>
-        <c:axId val="47176895"/>
+        <c:axId val="43782982"/>
+        <c:axId val="68731025"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="2262243"/>
+        <c:axId val="43782982"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2802,7 +2871,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47176895"/>
+        <c:crossAx val="68731025"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2810,7 +2879,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="47176895"/>
+        <c:axId val="68731025"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2886,7 +2955,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2262243"/>
+        <c:crossAx val="43782982"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3858,7 +3927,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>327</v>
+        <v>345</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3867,7 +3936,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>328</v>
+        <v>346</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3876,16 +3945,16 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>329</v>
+        <v>347</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>330</v>
+        <v>348</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>331</v>
+        <v>349</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>4</v>
@@ -3893,13 +3962,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>332</v>
+        <v>350</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>333</v>
+        <v>351</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>334</v>
+        <v>352</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>139</v>
@@ -3911,13 +3980,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>335</v>
+        <v>353</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>336</v>
+        <v>354</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>91</v>
@@ -3929,13 +3998,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>335</v>
+        <v>353</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>338</v>
+        <v>356</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>339</v>
+        <v>357</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>117</v>
@@ -3947,13 +4016,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>335</v>
+        <v>353</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>340</v>
+        <v>358</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>341</v>
+        <v>359</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>99</v>
@@ -3965,16 +4034,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>342</v>
+        <v>360</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>343</v>
+        <v>361</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>341</v>
+        <v>359</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>344</v>
+        <v>362</v>
       </c>
       <c r="E8" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C8,FIND(",",C8&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -3983,13 +4052,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>345</v>
+        <v>363</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>295</v>
+        <v>307</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>346</v>
+        <v>364</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>135</v>
@@ -4001,16 +4070,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>347</v>
+        <v>365</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>348</v>
+        <v>366</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>349</v>
+        <v>367</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>350</v>
+        <v>368</v>
       </c>
       <c r="E10" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C10,FIND(",",C10&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4019,16 +4088,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>351</v>
+        <v>369</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>352</v>
+        <v>370</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>353</v>
+        <v>371</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>354</v>
+        <v>372</v>
       </c>
       <c r="E11" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C11,FIND(",",C11&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4037,13 +4106,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>355</v>
+        <v>373</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>356</v>
+        <v>374</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>357</v>
+        <v>375</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>125</v>
@@ -4055,16 +4124,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>358</v>
+        <v>376</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>359</v>
+        <v>377</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>360</v>
+        <v>378</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>361</v>
+        <v>379</v>
       </c>
       <c r="E13" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C13,FIND(",",C13&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4073,16 +4142,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>362</v>
+        <v>380</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>363</v>
+        <v>381</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>364</v>
+        <v>382</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>365</v>
+        <v>383</v>
       </c>
       <c r="E14" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C14,FIND(",",C14&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4091,13 +4160,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>366</v>
+        <v>384</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>367</v>
+        <v>385</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>368</v>
+        <v>386</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>133</v>
@@ -4109,16 +4178,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>369</v>
+        <v>387</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>370</v>
+        <v>388</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>357</v>
+        <v>375</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>371</v>
+        <v>389</v>
       </c>
       <c r="E16" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C16,FIND(",",C16&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4127,16 +4196,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>372</v>
+        <v>390</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>373</v>
+        <v>391</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>374</v>
+        <v>392</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>375</v>
+        <v>393</v>
       </c>
       <c r="E17" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C17,FIND(",",C17&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4145,13 +4214,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>376</v>
+        <v>394</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>377</v>
+        <v>395</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>378</v>
+        <v>396</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>111</v>
@@ -4163,13 +4232,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>379</v>
+        <v>397</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>380</v>
+        <v>398</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>381</v>
+        <v>399</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>127</v>
@@ -4181,16 +4250,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>382</v>
+        <v>400</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>383</v>
+        <v>401</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>384</v>
+        <v>402</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>385</v>
+        <v>403</v>
       </c>
       <c r="E20" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C20,FIND(",",C20&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4199,16 +4268,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>386</v>
+        <v>404</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>387</v>
+        <v>405</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>388</v>
+        <v>406</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>389</v>
+        <v>407</v>
       </c>
       <c r="E21" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C21,FIND(",",C21&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4217,16 +4286,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>390</v>
+        <v>408</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>391</v>
+        <v>409</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>392</v>
+        <v>410</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>393</v>
+        <v>411</v>
       </c>
       <c r="E22" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C22,FIND(",",C22&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
@@ -4288,39 +4357,39 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>394</v>
+        <v>412</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>395</v>
+        <v>413</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>396</v>
+        <v>414</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>397</v>
+        <v>415</v>
       </c>
       <c r="B4" s="5" t="str">
-        <f aca="false">COUNTIF('Sprint Backlog'!$F$4:$F$39,"Terminado")&amp;" de "&amp;COUNTA('Sprint Backlog'!$A$4:$A$39)</f>
-        <v>32 de 36</v>
+        <f aca="false">COUNTIF('Sprint Backlog'!$F$4:$F$42,"Terminado")&amp;" de "&amp;COUNTA('Sprint Backlog'!$A$4:$A$42)</f>
+        <v>35 de 39</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>398</v>
+        <v>416</v>
       </c>
       <c r="B5" s="5" t="str">
-        <f aca="false">SUMIF('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$G$4:$G$39)&amp;" de "&amp;'Sprint Backlog'!$G$41&amp;" hrs"</f>
-        <v>150 de 165 hrs</v>
+        <f aca="false">SUMIF('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$G$4:$G$42)&amp;" de "&amp;'Sprint Backlog'!$G$44&amp;" hrs"</f>
+        <v>157 de 172 hrs</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>399</v>
+        <v>417</v>
       </c>
       <c r="B6" s="5" t="str">
         <f aca="false">COUNTIF('Feature Log'!$C$4:$C$29,"Terminado")&amp;" de "&amp;COUNTA('Feature Log'!$A$4:$A$29)</f>
@@ -4329,60 +4398,60 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>400</v>
+        <v>418</v>
       </c>
       <c r="B7" s="5" t="str">
-        <f aca="false">COUNTIF(Buglist!$E$4:$E$17,"Corregido")&amp;" de "&amp;COUNTA(Buglist!$A$4:$A$17)</f>
-        <v>13 de 14</v>
+        <f aca="false">COUNTIF(Buglist!$E$4:$E$18,"Corregido")&amp;" de "&amp;COUNTA(Buglist!$A$4:$A$18)</f>
+        <v>14 de 15</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>401</v>
+        <v>419</v>
       </c>
       <c r="B8" s="5" t="str">
-        <f aca="false">COUNTIF('Pruebas Alfa'!$G$4:$G$17,"Aprobada")&amp;" de "&amp;COUNTA('Pruebas Alfa'!$A$4:$A$17)</f>
-        <v>9 de 14</v>
+        <f aca="false">COUNTIF('Pruebas Alfa'!$G$4:$G$18,"Aprobada")&amp;" de "&amp;COUNTA('Pruebas Alfa'!$A$4:$A$18)</f>
+        <v>10 de 15</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>402</v>
+        <v>420</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>403</v>
+        <v>421</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>404</v>
+        <v>422</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>405</v>
+        <v>423</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>406</v>
+        <v>424</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>407</v>
+        <v>425</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>408</v>
+        <v>426</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>409</v>
+        <v>427</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>410</v>
+        <v>428</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>411</v>
+        <v>429</v>
       </c>
     </row>
   </sheetData>
@@ -4603,7 +4672,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -5614,12 +5683,14 @@
         <v>88</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>62</v>
+        <v>35</v>
       </c>
       <c r="G36" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H36" s="4"/>
+      <c r="H36" s="6" t="n">
+        <v>46308</v>
+      </c>
       <c r="I36" s="4"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5703,31 +5774,118 @@
         <v>46302</v>
       </c>
     </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B40" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>46308</v>
+      </c>
+      <c r="I40" s="6" t="n">
+        <v>46308</v>
+      </c>
+    </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F41" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="G41" s="8" t="n">
-        <f aca="false">SUM(G4:G39)</f>
+      <c r="A41" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B41" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H41" s="6" t="n">
+        <v>46308</v>
+      </c>
+      <c r="I41" s="6" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B42" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H42" s="6" t="n">
+        <v>46308</v>
+      </c>
+      <c r="I42" s="6" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F44" s="8" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F42" s="8" t="s">
-        <v>160</v>
-      </c>
-      <c r="G42" s="8" t="str">
-        <f aca="false">COUNTIF(F4:F39,"Terminado")&amp;" de "&amp;COUNTA(A4:A39)</f>
-        <v>32 de 36</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F43" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="G43" s="9" t="n">
-        <f aca="false">SUMIF(F4:F39,"Terminado",G4:G39)/G41</f>
-        <v>0.909090909090909</v>
+      <c r="G44" s="8" t="n">
+        <f aca="false">SUM(G4:G42)</f>
+        <v>172</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F45" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="G45" s="8" t="str">
+        <f aca="false">COUNTIF(F4:F42,"Terminado")&amp;" de "&amp;COUNTA(A4:A42)</f>
+        <v>35 de 39</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F46" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="G46" s="9" t="n">
+        <f aca="false">SUMIF(F4:F42,"Terminado",G4:G42)/G44</f>
+        <v>0.912790697674419</v>
       </c>
     </row>
   </sheetData>
@@ -5735,7 +5893,7 @@
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F4:F39">
+  <conditionalFormatting sqref="F4:F42">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminado"</formula>
     </cfRule>
@@ -5762,7 +5920,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F4:F39" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F4:F42" type="list">
       <formula1>"Terminado,En desarrollo,Planeado"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5782,7 +5940,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -5791,7 +5949,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5799,7 +5957,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5807,16 +5965,16 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5824,13 +5982,13 @@
         <v>46284</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5838,13 +5996,13 @@
         <v>46295</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5852,13 +6010,13 @@
         <v>46299</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5866,13 +6024,13 @@
         <v>46300</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5880,13 +6038,27 @@
         <v>46302</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>182</v>
+        <v>188</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -5919,14 +6091,14 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5934,10 +6106,10 @@
         <v>4</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5981,7 +6153,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="B7" s="13" t="n">
         <f aca="false">COUNTIF('Feature Log'!$C$4:$C$29,A7)</f>
@@ -5994,7 +6166,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="B8" s="15" t="n">
         <f aca="false">SUM(B4:B7)</f>
@@ -6032,7 +6204,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6040,7 +6212,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6050,16 +6222,16 @@
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6067,16 +6239,16 @@
         <v>46284</v>
       </c>
       <c r="B4" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A4)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>165</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A4)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>172</v>
       </c>
       <c r="C4" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$41-SUMIFS('Sprint Backlog'!$G$4:$G$39,'Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A4)</f>
-        <v>165</v>
+        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A4)</f>
+        <v>172</v>
       </c>
       <c r="D4" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-COUNTIFS('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A4)</f>
-        <v>36</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A4)</f>
+        <v>39</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6084,16 +6256,16 @@
         <v>46288</v>
       </c>
       <c r="B5" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A5)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>148.9</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A5)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>155.2</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$41-SUMIFS('Sprint Backlog'!$G$4:$G$39,'Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A5)</f>
-        <v>165</v>
+        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A5)</f>
+        <v>172</v>
       </c>
       <c r="D5" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-COUNTIFS('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A5)</f>
-        <v>36</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A5)</f>
+        <v>39</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6101,16 +6273,16 @@
         <v>46291</v>
       </c>
       <c r="B6" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A6)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>136.8</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A6)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>142.6</v>
       </c>
       <c r="C6" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$41-SUMIFS('Sprint Backlog'!$G$4:$G$39,'Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A6)</f>
-        <v>165</v>
+        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A6)</f>
+        <v>172</v>
       </c>
       <c r="D6" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-COUNTIFS('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A6)</f>
-        <v>36</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A6)</f>
+        <v>39</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6118,16 +6290,16 @@
         <v>46295</v>
       </c>
       <c r="B7" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A7)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>120.7</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A7)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>125.9</v>
       </c>
       <c r="C7" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$41-SUMIFS('Sprint Backlog'!$G$4:$G$39,'Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A7)</f>
-        <v>127</v>
+        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A7)</f>
+        <v>134</v>
       </c>
       <c r="D7" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-COUNTIFS('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A7)</f>
-        <v>29</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A7)</f>
+        <v>32</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6135,16 +6307,16 @@
         <v>46299</v>
       </c>
       <c r="B8" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A8)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>104.6</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A8)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>109.1</v>
       </c>
       <c r="C8" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$41-SUMIFS('Sprint Backlog'!$G$4:$G$39,'Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A8)</f>
-        <v>74</v>
+        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A8)</f>
+        <v>81</v>
       </c>
       <c r="D8" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-COUNTIFS('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A8)</f>
-        <v>20</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A8)</f>
+        <v>23</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6152,16 +6324,16 @@
         <v>46300</v>
       </c>
       <c r="B9" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A9)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>100.6</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A9)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>104.9</v>
       </c>
       <c r="C9" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$41-SUMIFS('Sprint Backlog'!$G$4:$G$39,'Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A9)</f>
-        <v>24</v>
+        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A9)</f>
+        <v>31</v>
       </c>
       <c r="D9" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-COUNTIFS('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A9)</f>
-        <v>8</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A9)</f>
+        <v>11</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6169,36 +6341,42 @@
         <v>46302</v>
       </c>
       <c r="B10" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A10)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>92.6</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A10)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>96.5</v>
       </c>
       <c r="C10" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$41-SUMIFS('Sprint Backlog'!$G$4:$G$39,'Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A10)</f>
-        <v>15</v>
+        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A10)</f>
+        <v>22</v>
       </c>
       <c r="D10" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-COUNTIFS('Sprint Backlog'!$F$4:$F$39,"Terminado",'Sprint Backlog'!$I$4:$I$39,"&lt;="&amp;A10)</f>
-        <v>4</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A10)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="n">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B11" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A11)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>64.4</v>
-      </c>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
+        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A11)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>71.3</v>
+      </c>
+      <c r="C11" s="13" t="n">
+        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A11)</f>
+        <v>15</v>
+      </c>
+      <c r="D11" s="13" t="n">
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A11)</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="n">
         <v>46316</v>
       </c>
       <c r="B12" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A12)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>36.2</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A12)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>37.8</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
@@ -6208,8 +6386,8 @@
         <v>46323</v>
       </c>
       <c r="B13" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A13)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>8</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A13)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>8.4</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
@@ -6219,7 +6397,7 @@
         <v>46325</v>
       </c>
       <c r="B14" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$41*('Sprint Plan'!$D$5-A14)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A14)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
         <v>0</v>
       </c>
       <c r="C14" s="13"/>
@@ -6246,7 +6424,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -6256,25 +6434,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6284,10 +6462,10 @@
       </c>
       <c r="B4" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D4</f>
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C4" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-B4</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B4</f>
         <v>0</v>
       </c>
     </row>
@@ -6298,10 +6476,10 @@
       </c>
       <c r="B5" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D5</f>
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-B5</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B5</f>
         <v>0</v>
       </c>
     </row>
@@ -6312,10 +6490,10 @@
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D6</f>
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C6" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-B6</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B6</f>
         <v>0</v>
       </c>
     </row>
@@ -6326,10 +6504,10 @@
       </c>
       <c r="B7" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D7</f>
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C7" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-B7</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B7</f>
         <v>7</v>
       </c>
     </row>
@@ -6340,10 +6518,10 @@
       </c>
       <c r="B8" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D8</f>
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C8" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-B8</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B8</f>
         <v>16</v>
       </c>
     </row>
@@ -6354,10 +6532,10 @@
       </c>
       <c r="B9" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D9</f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C9" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-B9</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B9</f>
         <v>28</v>
       </c>
     </row>
@@ -6368,11 +6546,25 @@
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D10</f>
+        <v>7</v>
+      </c>
+      <c r="C10" s="13" t="n">
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B10</f>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17" t="n">
+        <f aca="false">'Burn-down Chart'!A11</f>
+        <v>46308</v>
+      </c>
+      <c r="B11" s="13" t="n">
+        <f aca="false">'Burn-down Chart'!D11</f>
         <v>4</v>
       </c>
-      <c r="C10" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$39)-B10</f>
-        <v>32</v>
+      <c r="C11" s="13" t="n">
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B11</f>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -6395,7 +6587,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -6410,7 +6602,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6422,7 +6614,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6434,16 +6626,16 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>4</v>
@@ -6452,27 +6644,27 @@
         <v>2</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>15</v>
@@ -6481,24 +6673,24 @@
         <v>46299</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>14</v>
@@ -6507,24 +6699,24 @@
         <v>46300</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>19</v>
@@ -6533,24 +6725,24 @@
         <v>46300</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>15</v>
@@ -6559,24 +6751,24 @@
         <v>46300</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>17</v>
@@ -6585,24 +6777,24 @@
         <v>46300</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>11</v>
@@ -6611,24 +6803,24 @@
         <v>46300</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>18</v>
@@ -6637,24 +6829,24 @@
         <v>46300</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>13</v>
@@ -6663,24 +6855,24 @@
         <v>46300</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>19</v>
@@ -6689,24 +6881,24 @@
         <v>46300</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="F13" s="4" t="n">
         <v>22</v>
@@ -6715,24 +6907,24 @@
         <v>46300</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>17</v>
@@ -6741,24 +6933,24 @@
         <v>46300</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>11</v>
@@ -6767,24 +6959,24 @@
         <v>46302</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="F16" s="4" t="n">
         <v>20</v>
@@ -6793,24 +6985,24 @@
         <v>46302</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
       <c r="F17" s="4" t="n">
         <v>21</v>
@@ -6819,16 +7011,42 @@
         <v>46302</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D19" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="E19" s="8" t="str">
-        <f aca="false">COUNTIF(E4:E17,"Corregido")&amp;" de "&amp;COUNTA(A4:A17)</f>
-        <v>13 de 14</v>
+        <v>218</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>46308</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D20" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="E20" s="8" t="str">
+        <f aca="false">COUNTIF(E4:E18,"Corregido")&amp;" de "&amp;COUNTA(A4:A18)</f>
+        <v>14 de 15</v>
       </c>
     </row>
   </sheetData>
@@ -6836,7 +7054,7 @@
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E4:E17">
+  <conditionalFormatting sqref="E4:E18">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminado"</formula>
     </cfRule>
@@ -6877,7 +7095,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -6891,7 +7109,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6902,7 +7120,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6913,22 +7131,22 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>4</v>
@@ -6936,325 +7154,350 @@
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>275</v>
+        <v>287</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>20</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="D7" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="G7" s="4" t="s">
         <v>277</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>278</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>270</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>279</v>
+        <v>291</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>19</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>281</v>
+        <v>293</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>17</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>285</v>
+        <v>297</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>287</v>
+        <v>299</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>289</v>
+        <v>301</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>13</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>292</v>
+        <v>304</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>293</v>
+        <v>305</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>16</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>295</v>
+        <v>307</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>298</v>
+        <v>310</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>302</v>
+        <v>314</v>
       </c>
       <c r="F12" s="5"/>
       <c r="G12" s="4" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>305</v>
+        <v>317</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>306</v>
+        <v>318</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>307</v>
+        <v>319</v>
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="4" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>308</v>
+        <v>320</v>
       </c>
       <c r="B14" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>309</v>
+        <v>321</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>312</v>
+        <v>324</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>313</v>
+        <v>325</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>11</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>314</v>
+        <v>326</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>316</v>
+        <v>328</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>318</v>
+        <v>330</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>23</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>319</v>
+        <v>331</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
       <c r="F16" s="5"/>
       <c r="G16" s="4" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>24</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>324</v>
+        <v>336</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="F17" s="5"/>
+        <v>337</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>338</v>
+      </c>
       <c r="G17" s="4" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F19" s="8" t="s">
-        <v>326</v>
-      </c>
-      <c r="G19" s="8" t="str">
-        <f aca="false">COUNTIF(G4:G17,"Aprobada")&amp;" de "&amp;COUNTA(A4:A17)</f>
-        <v>9 de 14</v>
+        <v>315</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F20" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="G20" s="8" t="str">
+        <f aca="false">COUNTIF(G4:G18,"Aprobada")&amp;" de "&amp;COUNTA(A4:A18)</f>
+        <v>10 de 15</v>
       </c>
     </row>
   </sheetData>
@@ -7262,7 +7505,7 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G4:G17">
+  <conditionalFormatting sqref="G4:G18">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminado"</formula>
     </cfRule>
@@ -7292,7 +7535,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G4:G17" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G4:G18" type="list">
       <formula1>"Aprobada,Fallida,Pendiente"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Formato de Pruebas Beta y hoja de resultados para el Sprint 3
</commit_message>
<xml_diff>
--- a/Documentacion/Producto2/PérezAlcántaraAlejandro_producción_10D_Sprint2.xlsx
+++ b/Documentacion/Producto2/PérezAlcántaraAlejandro_producción_10D_Sprint2.xlsx
@@ -19,6 +19,7 @@
     <sheet name="Pruebas Alfa" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="Matriz GDD" sheetId="10" state="visible" r:id="rId12"/>
     <sheet name="Sprint Review" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="Pruebas Beta" sheetId="12" state="visible" r:id="rId14"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="463">
   <si>
     <t xml:space="preserve">FEATURE LOG - ECOS DEL GRIMORIO (actualizado al Sprint 2)</t>
   </si>
@@ -605,7 +606,7 @@
     <t xml:space="preserve">Corregir a Lira flotando, controles de teclado para laptop, manual del jugador y generar el .exe.</t>
   </si>
   <si>
-    <t xml:space="preserve">El profesor notó que Lira flota sobre el suelo (B-015).</t>
+    <t xml:space="preserve">En la revisión de avance en clase se vio que Lira flota sobre el suelo (B-015).</t>
   </si>
   <si>
     <t xml:space="preserve">PROJECT CHART - Estado general del proyecto</t>
@@ -818,7 +819,7 @@
     <t xml:space="preserve">B-015</t>
   </si>
   <si>
-    <t xml:space="preserve">El profesor notó que Lira a veces flota sobre el suelo y las plataformas.</t>
+    <t xml:space="preserve">Lira a veces flota sobre el suelo y las plataformas (se vio en la revisión de avance en clase).</t>
   </si>
   <si>
     <t xml:space="preserve">La imagen de Lira tiene 17% de espacio transparente bajo los pies y el collider se calculaba con la imagen completa. Ahora EditorHelpers.MargenesTransparentes() lee el PNG y ajusta el collider y el GroundCheck a los pies reales.</t>
@@ -1320,6 +1321,105 @@
   </si>
   <si>
     <t xml:space="preserve">30 de octubre de 2026 (entrega del Producto 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRUEBAS BETA - SPRINT 3 (31 oct - 20 nov, 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Una fila por cada persona que prueba el juego, copiada de su formato de Pruebas Beta. Calificaciones del 1 (malo) al 5 (excelente). Los errores nuevos se pasan al Buglist con su BugID.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jugador(a)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jugó con</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ala a la que llegó</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minutos jugados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diversión (1-5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Controles claros (1-5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dificultad (1-5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lo que más le gustó</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lo que no entendió</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Errores (BugID)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PB-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personas que probaron:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Promedio diversión:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Promedio controles:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Promedio dificultad:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terminaron el juego:</t>
   </si>
 </sst>
 </file>
@@ -1477,7 +1577,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1552,6 +1652,10 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2303,11 +2407,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="6751934"/>
-        <c:axId val="62335594"/>
+        <c:axId val="15420128"/>
+        <c:axId val="71400424"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="6751934"/>
+        <c:axId val="15420128"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2373,7 +2477,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62335594"/>
+        <c:crossAx val="71400424"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2381,7 +2485,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="62335594"/>
+        <c:axId val="71400424"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2457,7 +2561,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6751934"/>
+        <c:crossAx val="15420128"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2801,11 +2905,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="43782982"/>
-        <c:axId val="68731025"/>
+        <c:axId val="63924923"/>
+        <c:axId val="22403101"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="43782982"/>
+        <c:axId val="63924923"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2871,7 +2975,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68731025"/>
+        <c:crossAx val="22403101"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2879,7 +2983,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="68731025"/>
+        <c:axId val="22403101"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2955,7 +3059,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43782982"/>
+        <c:crossAx val="63924923"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4468,6 +4572,486 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:N24"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="B4" s="6"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="B5" s="6"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="B6" s="6"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>447</v>
+      </c>
+      <c r="B8" s="6"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="B9" s="6"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="B10" s="6"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="B11" s="6"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="B12" s="6"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>452</v>
+      </c>
+      <c r="B13" s="6"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>453</v>
+      </c>
+      <c r="B14" s="6"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="B15" s="6"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>455</v>
+      </c>
+      <c r="B16" s="6"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="4"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>456</v>
+      </c>
+      <c r="B17" s="6"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="4"/>
+      <c r="N17" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>457</v>
+      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F20" s="8" t="s">
+        <v>458</v>
+      </c>
+      <c r="H20" s="19" t="n">
+        <f aca="false">COUNTA(C4:C18)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F21" s="8" t="s">
+        <v>459</v>
+      </c>
+      <c r="H21" s="0" t="str">
+        <f aca="false">IF(COUNT(H4:H18)=0,"",ROUND(AVERAGE(H4:H18),1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F22" s="8" t="s">
+        <v>460</v>
+      </c>
+      <c r="H22" s="0" t="str">
+        <f aca="false">IF(COUNT(I4:I18)=0,"",ROUND(AVERAGE(I4:I18),1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F23" s="8" t="s">
+        <v>461</v>
+      </c>
+      <c r="H23" s="0" t="str">
+        <f aca="false">IF(COUNT(J4:J18)=0,"",ROUND(AVERAGE(J4:J18),1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F24" s="8" t="s">
+        <v>462</v>
+      </c>
+      <c r="H24" s="19" t="n">
+        <f aca="false">COUNTIF(F4:F18,"Terminó el juego")</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A2:N2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="N4:N18">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"Terminado"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"En desarrollo"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>"Planeado"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"Corregido"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"Aprobada"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Por verificar"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Pendiente"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>"Abierto"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="5">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D4:D18" type="list">
+      <formula1>"Cerrada,Abierta"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E4:E18" type="list">
+      <formula1>"Teclado,Control PS4,Control Xbox"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F4:F18" type="list">
+      <formula1>"Aprendizaje,Fuego,Hielo,Viento,Corazón,Terminó el juego"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N4:N18" type="list">
+      <formula1>"Pendiente,Registrada,Atendida"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H4:J18" type="whole">
+      <formula1>1</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">

</xml_diff>

<commit_message>
Saltar nivel, versión 1.0 del juego, manual actualizado y documentos del Sprint 3
</commit_message>
<xml_diff>
--- a/Documentacion/Producto2/PérezAlcántaraAlejandro_producción_10D_Sprint2.xlsx
+++ b/Documentacion/Producto2/PérezAlcántaraAlejandro_producción_10D_Sprint2.xlsx
@@ -31,12 +31,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="506">
   <si>
     <t xml:space="preserve">FEATURE LOG - ECOS DEL GRIMORIO (actualizado al Sprint 2)</t>
   </si>
   <si>
-    <t xml:space="preserve">Los features 1 a 14 vienen del Feature Log inicial (GDD 3.1); del 15 al 26 se agregaron en el Sprint 2 para cubrir secciones del GDD que no tenían feature.</t>
+    <t xml:space="preserve">Los features 1 a 14 vienen del Feature Log inicial (GDD 3.1); del 15 al 26 se agregaron en el Sprint 2 para cubrir secciones del GDD que no tenían feature; el 27 salió de las pruebas.</t>
   </si>
   <si>
     <t xml:space="preserve">Featureid</t>
@@ -174,7 +174,7 @@
     <t xml:space="preserve">Música, efectos de sonido y voces (2.17)</t>
   </si>
   <si>
-    <t xml:space="preserve">9 pistas, 29 efectos y voces por personaje</t>
+    <t xml:space="preserve">9 pistas, 41 efectos (12 agregados el 15 oct) y voces por personaje</t>
   </si>
   <si>
     <t xml:space="preserve">Control de PS4 / Xbox y vibración (2.4)</t>
@@ -207,13 +207,13 @@
     <t xml:space="preserve">2-3</t>
   </si>
   <si>
-    <t xml:space="preserve">Menú Ecos del Grimorio &gt; Compilar juego (.exe)</t>
+    <t xml:space="preserve">Menú Ecos del Grimorio &gt; Compilar juego (.exe). Primera compilación el 13 oct y versión 1.0 el 20 oct; falta probarlo en otra computadora</t>
   </si>
   <si>
     <t xml:space="preserve">Documentación del Producto 2 (producción y evidencias)</t>
   </si>
   <si>
-    <t xml:space="preserve">Documento Word/PDF y este libro de Excel</t>
+    <t xml:space="preserve">Documento Word/PDF, manual del jugador y este libro de Excel</t>
   </si>
   <si>
     <t xml:space="preserve">Pruebas Beta y reporte Postmortem</t>
@@ -225,6 +225,12 @@
     <t xml:space="preserve">Jugadores externos; plantilla de Postmortem de Huddle</t>
   </si>
   <si>
+    <t xml:space="preserve">Ayudas al jugador: ayuda para apuntar, sentido arcano y saltar nivel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agregado después de las pruebas del 14 y 15 de octubre y de la revisión en clase</t>
+  </si>
+  <si>
     <t xml:space="preserve">SPRINT PLAN - ECOS DEL GRIMORIO (replaneado en el Sprint 2)</t>
   </si>
   <si>
@@ -528,6 +534,48 @@
     <t xml:space="preserve">Manual del jugador en PDF</t>
   </si>
   <si>
+    <t xml:space="preserve">T40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ayuda para apuntar: el hechizo sigue al enemigo más cercano a la mira (opción en Opciones)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aves de Tormenta: aviso antes de la picada, descanso después y menos empuje (B-016)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giro de Lira hacia donde camina con animación (B-017)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sentido arcano: chispas, tintineo y aviso cerca de secretos (B-018)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 efectos de sonido nuevos (lanzar, sin maná, quejido, graznido, caídas, latido, etc.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saltar nivel: opción en la pausa y mantener N o L3 + R3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compilar la versión 1.0 del .exe y actualizar el manual</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total horas:</t>
   </si>
   <si>
@@ -609,6 +657,24 @@
     <t xml:space="preserve">En la revisión de avance en clase se vio que Lira flota sobre el suelo (B-015).</t>
   </si>
   <si>
+    <t xml:space="preserve">Primer .exe, manual y controles para laptop. Jugué el Ala de Viento con el control de PS4.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ayuda para apuntar, aves con aviso, giro de Lira, sentido arcano y sonidos nuevos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Las aves son difíciles de atinar y empujan a Lira al vacío (B-016); Lira no se voltea bien (B-017); no se encuentran los secretos (B-018). Unity se quedaba cargando al abrir el proyecto (se resolvió cerrando procesos).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mejoras del 15 de octubre probadas; en la revisión en clase el juego gustó.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saltar nivel para la presentación, versión 1.0 del .exe, manual actualizado y preparar el Sprint 3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ninguno.</t>
+  </si>
+  <si>
     <t xml:space="preserve">PROJECT CHART - Estado general del proyecto</t>
   </si>
   <si>
@@ -825,6 +891,33 @@
     <t xml:space="preserve">La imagen de Lira tiene 17% de espacio transparente bajo los pies y el collider se calculaba con la imagen completa. Ahora EditorHelpers.MargenesTransparentes() lee el PNG y ajusta el collider y el GroundCheck a los pies reales.</t>
   </si>
   <si>
+    <t xml:space="preserve">B-016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En el Ala de Viento es difícil atinarle a las Aves de Tormenta y empujan a Lira al vacío.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se mueven con ruido de Perlin y se lanzan sin aviso. Ahora tiemblan y graznan 0.55 s antes de la picada, descansan 0.8 s después y empujan con fuerza 5 en vez de 9. Además se agregó la ayuda para apuntar (SpellCaster.BuscarObjetivo + SpellProjectile.Seguir).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Al caminar hacia atrás Lira no parece voltearse.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El dibujo original mira un poco a la izquierda y el código volteaba el sprite como si mirara a la derecha. Campo arteMiraALaDerecha en PlayerController y giro animado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B-018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No se sabe dónde están las Páginas Perdidas ni los secretos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No había ninguna pista cerca de ellos. SentidoArcano.cs muestra chispas, un tintineo y un aviso a menos de 7 unidades.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Corregidos:</t>
   </si>
   <si>
@@ -1065,6 +1158,30 @@
     <t xml:space="preserve">Flotaba (B-015). Corregido.</t>
   </si>
   <si>
+    <t xml:space="preserve">PA-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saltar nivel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En cada ala mantener N (o L3 + R3) 1.5 s, y probar Pausa &gt; Saltar nivel.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pasa a la siguiente ala con el hechizo que tocaba; en el Corazón pasa al final. No da logros.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PA-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ayuda para apuntar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disparar a las Aves de Tormenta con y sin la opción activada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Con la opción, el hechizo sigue al ave; sin ella, va en línea recta.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Aprobadas:</t>
   </si>
   <si>
@@ -1266,10 +1383,22 @@
     <t xml:space="preserve">24</t>
   </si>
   <si>
-    <t xml:space="preserve">T30, T33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SPRINT REVIEW - SPRINT 2 (avance al 13 de octubre de 2026)</t>
+    <t xml:space="preserve">T30, T33, T46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.4 / 2.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ayudas al jugador y opción de ayuda para apuntar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T40, T43, T45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPRINT REVIEW - SPRINT 2 (avance al 20 de octubre de 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Meta del sprint</t>
@@ -1296,7 +1425,7 @@
     <t xml:space="preserve">Demostración</t>
   </si>
   <si>
-    <t xml:space="preserve">Partida desde el menú hasta el Ala de Fuego con el control de PS4: diálogo con la Maestra Sable, combate, sala secreta, pantalla de resultados y Opciones.</t>
+    <t xml:space="preserve">Partida con el .exe y el control de PS4: diálogo con la Maestra Sable, combate, sala secreta, pantalla de resultados, Opciones y saltar nivel para mostrar las cinco alas y el final.</t>
   </si>
   <si>
     <t xml:space="preserve">¿Qué salió bien?</t>
@@ -1308,7 +1437,7 @@
     <t xml:space="preserve">¿Qué salió mal?</t>
   </si>
   <si>
-    <t xml:space="preserve">Varias fallas solo aparecieron al jugar con el control (sonido, textos fuera del marco, final del juego). El Burn-down muestra que la mayor parte del trabajo se concentró en pocos días.</t>
+    <t xml:space="preserve">Varias fallas solo aparecieron al jugar con el control (sonido, textos fuera del marco, final del juego) o en la revisión en clase (Lira flotando). El Ala de Viento quedó muy difícil por las aves. El Burn-down muestra que la mayor parte del trabajo se concentró en pocos días.</t>
   </si>
   <si>
     <t xml:space="preserve">Ajustes para el Sprint 3</t>
@@ -2022,10 +2151,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>22</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1</c:v>
@@ -2187,9 +2316,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Burn-down Chart'!$A$4:$A$14</c:f>
+              <c:f>'Burn-down Chart'!$A$4:$A$15</c:f>
               <c:strCache>
-                <c:ptCount val="11"/>
+                <c:ptCount val="12"/>
                 <c:pt idx="0">
                   <c:v>19/09</c:v>
                 </c:pt>
@@ -2215,12 +2344,15 @@
                   <c:v>13/10</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>21/10</c:v>
+                  <c:v>15/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>28/10</c:v>
+                  <c:v>20/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>25/10</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>30/10</c:v>
                 </c:pt>
               </c:strCache>
@@ -2228,41 +2360,44 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Burn-down Chart'!$B$4:$B$14</c:f>
+              <c:f>'Burn-down Chart'!$B$4:$B$15</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>172</c:v>
+                  <c:v>187</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>155.2</c:v>
+                  <c:v>168.8</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>142.6</c:v>
+                  <c:v>155.1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>125.9</c:v>
+                  <c:v>136.8</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>109.1</c:v>
+                  <c:v>118.6</c:v>
                 </c:pt>
                 <c:pt idx="5">
+                  <c:v>114</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>104.9</c:v>
                 </c:pt>
-                <c:pt idx="6">
-                  <c:v>96.5</c:v>
-                </c:pt>
                 <c:pt idx="7">
-                  <c:v>71.3</c:v>
+                  <c:v>77.5</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>37.8</c:v>
+                  <c:v>68.4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>8.4</c:v>
+                  <c:v>45.6</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>22.8</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -2325,9 +2460,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Burn-down Chart'!$A$4:$A$14</c:f>
+              <c:f>'Burn-down Chart'!$A$4:$A$15</c:f>
               <c:strCache>
-                <c:ptCount val="11"/>
+                <c:ptCount val="12"/>
                 <c:pt idx="0">
                   <c:v>19/09</c:v>
                 </c:pt>
@@ -2353,12 +2488,15 @@
                   <c:v>13/10</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>21/10</c:v>
+                  <c:v>15/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>28/10</c:v>
+                  <c:v>20/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>25/10</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>30/10</c:v>
                 </c:pt>
               </c:strCache>
@@ -2366,33 +2504,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Burn-down Chart'!$C$4:$C$14</c:f>
+              <c:f>'Burn-down Chart'!$C$4:$C$15</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>172</c:v>
+                  <c:v>187</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>172</c:v>
+                  <c:v>187</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>172</c:v>
+                  <c:v>187</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>134</c:v>
+                  <c:v>149</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>81</c:v>
+                  <c:v>96</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>31</c:v>
+                  <c:v>46</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>22</c:v>
+                  <c:v>37</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>15</c:v>
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2407,11 +2551,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="15420128"/>
-        <c:axId val="71400424"/>
+        <c:axId val="26128128"/>
+        <c:axId val="12110244"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="15420128"/>
+        <c:axId val="26128128"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2477,7 +2621,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71400424"/>
+        <c:crossAx val="12110244"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2485,7 +2629,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="71400424"/>
+        <c:axId val="12110244"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2561,7 +2705,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15420128"/>
+        <c:crossAx val="26128128"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2712,9 +2856,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Task Chart'!$A$4:$A$11</c:f>
+              <c:f>'Task Chart'!$A$4:$A$13</c:f>
               <c:strCache>
-                <c:ptCount val="8"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
                   <c:v>19/09</c:v>
                 </c:pt>
@@ -2738,39 +2882,51 @@
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>13/10</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>15/10</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>20/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Task Chart'!$B$4:$B$11</c:f>
+              <c:f>'Task Chart'!$B$4:$B$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>39</c:v>
                 </c:pt>
-                <c:pt idx="1">
-                  <c:v>39</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>39</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>32</c:v>
-                </c:pt>
                 <c:pt idx="4">
-                  <c:v>23</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>11</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>7</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4</c:v>
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2832,9 +2988,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Task Chart'!$A$4:$A$11</c:f>
+              <c:f>'Task Chart'!$A$4:$A$13</c:f>
               <c:strCache>
-                <c:ptCount val="8"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
                   <c:v>19/09</c:v>
                 </c:pt>
@@ -2858,16 +3014,22 @@
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>13/10</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>15/10</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>20/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Task Chart'!$C$4:$C$11</c:f>
+              <c:f>'Task Chart'!$C$4:$C$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="10"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -2890,7 +3052,13 @@
                   <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>35</c:v>
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>43</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2905,11 +3073,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="63924923"/>
-        <c:axId val="22403101"/>
+        <c:axId val="15060964"/>
+        <c:axId val="64371788"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="63924923"/>
+        <c:axId val="15060964"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2975,7 +3143,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22403101"/>
+        <c:crossAx val="64371788"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2983,7 +3151,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="22403101"/>
+        <c:axId val="64371788"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3059,7 +3227,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63924923"/>
+        <c:crossAx val="15060964"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3396,7 +3564,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -3807,7 +3975,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="n">
         <v>19</v>
       </c>
@@ -3907,7 +4075,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="n">
         <v>24</v>
       </c>
@@ -3935,7 +4103,7 @@
         <v>59</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="D28" s="4" t="n">
         <v>2</v>
@@ -3965,6 +4133,26 @@
       </c>
       <c r="F29" s="5" t="s">
         <v>63</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -3972,7 +4160,7 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
   </mergeCells>
-  <conditionalFormatting sqref="C4:C29">
+  <conditionalFormatting sqref="C4:C30">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminado"</formula>
     </cfRule>
@@ -3999,7 +4187,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C4:C29" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C4:C30" type="list">
       <formula1>"Terminado,En desarrollo,Planeado,Sin planear"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4019,7 +4207,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -4031,7 +4219,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>345</v>
+        <v>384</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4040,7 +4228,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>346</v>
+        <v>385</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4049,16 +4237,16 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>347</v>
+        <v>386</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>348</v>
+        <v>387</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>349</v>
+        <v>388</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>4</v>
@@ -4066,344 +4254,362 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>350</v>
+        <v>389</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>351</v>
+        <v>390</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>352</v>
+        <v>391</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E4" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C4,FIND(",",C4&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C4,FIND(",",C4&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>353</v>
+        <v>392</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>354</v>
+        <v>393</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>355</v>
+        <v>394</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E5" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C5,FIND(",",C5&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C5,FIND(",",C5&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>353</v>
+        <v>392</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>356</v>
+        <v>395</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>357</v>
+        <v>396</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E6" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C6,FIND(",",C6&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C6,FIND(",",C6&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>353</v>
+        <v>392</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>358</v>
+        <v>397</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>359</v>
+        <v>398</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E7" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C7,FIND(",",C7&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C7,FIND(",",C7&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>360</v>
+        <v>399</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>361</v>
+        <v>400</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>359</v>
+        <v>398</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>362</v>
+        <v>401</v>
       </c>
       <c r="E8" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C8,FIND(",",C8&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C8,FIND(",",C8&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>363</v>
+        <v>402</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>307</v>
+        <v>338</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>364</v>
+        <v>403</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E9" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C9,FIND(",",C9&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C9,FIND(",",C9&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>365</v>
+        <v>404</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>366</v>
+        <v>405</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>367</v>
+        <v>406</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>368</v>
+        <v>407</v>
       </c>
       <c r="E10" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C10,FIND(",",C10&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C10,FIND(",",C10&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>369</v>
+        <v>408</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>370</v>
+        <v>409</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>371</v>
+        <v>410</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>372</v>
+        <v>411</v>
       </c>
       <c r="E11" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C11,FIND(",",C11&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C11,FIND(",",C11&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>373</v>
+        <v>412</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>374</v>
+        <v>413</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>375</v>
+        <v>414</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E12" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C12,FIND(",",C12&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C12,FIND(",",C12&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>376</v>
+        <v>415</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>377</v>
+        <v>416</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>378</v>
+        <v>417</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>379</v>
+        <v>418</v>
       </c>
       <c r="E13" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C13,FIND(",",C13&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C13,FIND(",",C13&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>380</v>
+        <v>419</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>381</v>
+        <v>420</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>382</v>
+        <v>421</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>383</v>
+        <v>422</v>
       </c>
       <c r="E14" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C14,FIND(",",C14&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C14,FIND(",",C14&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>384</v>
+        <v>423</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>385</v>
+        <v>424</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>386</v>
+        <v>425</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E15" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C15,FIND(",",C15&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C15,FIND(",",C15&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>387</v>
+        <v>426</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>388</v>
+        <v>427</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>375</v>
+        <v>414</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>389</v>
+        <v>428</v>
       </c>
       <c r="E16" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C16,FIND(",",C16&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C16,FIND(",",C16&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>390</v>
+        <v>429</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>391</v>
+        <v>430</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>392</v>
+        <v>431</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>393</v>
+        <v>432</v>
       </c>
       <c r="E17" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C17,FIND(",",C17&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C17,FIND(",",C17&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>394</v>
+        <v>433</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>395</v>
+        <v>434</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>396</v>
+        <v>435</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E18" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C18,FIND(",",C18&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C18,FIND(",",C18&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>397</v>
+        <v>436</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>398</v>
+        <v>437</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>399</v>
+        <v>438</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E19" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C19,FIND(",",C19&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C19,FIND(",",C19&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>400</v>
+        <v>439</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>401</v>
+        <v>440</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>402</v>
+        <v>441</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>403</v>
+        <v>442</v>
       </c>
       <c r="E20" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C20,FIND(",",C20&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C20,FIND(",",C20&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>404</v>
+        <v>443</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>405</v>
+        <v>444</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>406</v>
+        <v>445</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>407</v>
+        <v>446</v>
       </c>
       <c r="E21" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C21,FIND(",",C21&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C21,FIND(",",C21&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>En desarrollo</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>408</v>
+        <v>447</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>409</v>
+        <v>448</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>410</v>
+        <v>449</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>411</v>
+        <v>450</v>
       </c>
       <c r="E22" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$29,MATCH(VALUE(LEFT(C22,FIND(",",C22&amp;",")-1)),'Feature Log'!$A$4:$A$29,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C22,FIND(",",C22&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
         <v>En desarrollo</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>453</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="E23" s="4" t="str">
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C23,FIND(",",C23&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <v>Terminado</v>
       </c>
     </row>
   </sheetData>
@@ -4411,7 +4617,7 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E4:E22">
+  <conditionalFormatting sqref="E4:E23">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminado"</formula>
     </cfRule>
@@ -4461,101 +4667,101 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>412</v>
+        <v>455</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>413</v>
+        <v>456</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>414</v>
+        <v>457</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>415</v>
+        <v>458</v>
       </c>
       <c r="B4" s="5" t="str">
-        <f aca="false">COUNTIF('Sprint Backlog'!$F$4:$F$42,"Terminado")&amp;" de "&amp;COUNTA('Sprint Backlog'!$A$4:$A$42)</f>
-        <v>35 de 39</v>
+        <f aca="false">COUNTIF('Sprint Backlog'!$F$4:$F$49,"Terminado")&amp;" de "&amp;COUNTA('Sprint Backlog'!$A$4:$A$49)</f>
+        <v>43 de 46</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>416</v>
+        <v>459</v>
       </c>
       <c r="B5" s="5" t="str">
-        <f aca="false">SUMIF('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$G$4:$G$42)&amp;" de "&amp;'Sprint Backlog'!$G$44&amp;" hrs"</f>
-        <v>157 de 172 hrs</v>
+        <f aca="false">SUMIF('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$G$4:$G$49)&amp;" de "&amp;'Sprint Backlog'!$G$51&amp;" hrs"</f>
+        <v>178 de 187 hrs</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>417</v>
+        <v>460</v>
       </c>
       <c r="B6" s="5" t="str">
-        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$29,"Terminado")&amp;" de "&amp;COUNTA('Feature Log'!$A$4:$A$29)</f>
-        <v>22 de 26</v>
+        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$30,"Terminado")&amp;" de "&amp;COUNTA('Feature Log'!$A$4:$A$30)</f>
+        <v>24 de 27</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>418</v>
+        <v>461</v>
       </c>
       <c r="B7" s="5" t="str">
-        <f aca="false">COUNTIF(Buglist!$E$4:$E$18,"Corregido")&amp;" de "&amp;COUNTA(Buglist!$A$4:$A$18)</f>
-        <v>14 de 15</v>
+        <f aca="false">COUNTIF(Buglist!$E$4:$E$21,"Corregido")&amp;" de "&amp;COUNTA(Buglist!$A$4:$A$21)</f>
+        <v>17 de 18</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>419</v>
+        <v>462</v>
       </c>
       <c r="B8" s="5" t="str">
-        <f aca="false">COUNTIF('Pruebas Alfa'!$G$4:$G$18,"Aprobada")&amp;" de "&amp;COUNTA('Pruebas Alfa'!$A$4:$A$18)</f>
-        <v>10 de 15</v>
+        <f aca="false">COUNTIF('Pruebas Alfa'!$G$4:$G$20,"Aprobada")&amp;" de "&amp;COUNTA('Pruebas Alfa'!$A$4:$A$20)</f>
+        <v>10 de 17</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>420</v>
+        <v>463</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>421</v>
+        <v>464</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>422</v>
+        <v>465</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>424</v>
+        <v>467</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>425</v>
+        <v>468</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>426</v>
+        <v>469</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>427</v>
+        <v>470</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>428</v>
+        <v>471</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>429</v>
+        <v>472</v>
       </c>
     </row>
   </sheetData>
@@ -4596,7 +4802,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>430</v>
+        <v>473</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4614,7 +4820,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>431</v>
+        <v>474</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4632,43 +4838,43 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>267</v>
+        <v>298</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>432</v>
+        <v>475</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>433</v>
+        <v>476</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>434</v>
+        <v>477</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>435</v>
+        <v>478</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>436</v>
+        <v>479</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>437</v>
+        <v>480</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>438</v>
+        <v>481</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>439</v>
+        <v>482</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>440</v>
+        <v>483</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>441</v>
+        <v>484</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>442</v>
+        <v>485</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>4</v>
@@ -4676,7 +4882,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>443</v>
+        <v>486</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="5"/>
@@ -4694,7 +4900,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>444</v>
+        <v>487</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="5"/>
@@ -4712,7 +4918,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>445</v>
+        <v>488</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="5"/>
@@ -4730,7 +4936,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>446</v>
+        <v>489</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="5"/>
@@ -4748,7 +4954,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>447</v>
+        <v>490</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="5"/>
@@ -4766,7 +4972,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>448</v>
+        <v>491</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="5"/>
@@ -4784,7 +4990,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>449</v>
+        <v>492</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="5"/>
@@ -4802,7 +5008,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>450</v>
+        <v>493</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="5"/>
@@ -4820,7 +5026,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>451</v>
+        <v>494</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="5"/>
@@ -4838,7 +5044,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>452</v>
+        <v>495</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="5"/>
@@ -4856,7 +5062,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>453</v>
+        <v>496</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="5"/>
@@ -4874,7 +5080,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>454</v>
+        <v>497</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="5"/>
@@ -4892,7 +5098,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>455</v>
+        <v>498</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="5"/>
@@ -4910,7 +5116,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>456</v>
+        <v>499</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="5"/>
@@ -4928,7 +5134,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>457</v>
+        <v>500</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="5"/>
@@ -4946,7 +5152,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F20" s="8" t="s">
-        <v>458</v>
+        <v>501</v>
       </c>
       <c r="H20" s="19" t="n">
         <f aca="false">COUNTA(C4:C18)</f>
@@ -4955,7 +5161,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F21" s="8" t="s">
-        <v>459</v>
+        <v>502</v>
       </c>
       <c r="H21" s="0" t="str">
         <f aca="false">IF(COUNT(H4:H18)=0,"",ROUND(AVERAGE(H4:H18),1))</f>
@@ -4964,7 +5170,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F22" s="8" t="s">
-        <v>460</v>
+        <v>503</v>
       </c>
       <c r="H22" s="0" t="str">
         <f aca="false">IF(COUNT(I4:I18)=0,"",ROUND(AVERAGE(I4:I18),1))</f>
@@ -4973,7 +5179,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F23" s="8" t="s">
-        <v>461</v>
+        <v>504</v>
       </c>
       <c r="H23" s="0" t="str">
         <f aca="false">IF(COUNT(J4:J18)=0,"",ROUND(AVERAGE(J4:J18),1))</f>
@@ -4982,7 +5188,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F24" s="8" t="s">
-        <v>462</v>
+        <v>505</v>
       </c>
       <c r="H24" s="19" t="n">
         <f aca="false">COUNTIF(F4:F18,"Terminó el juego")</f>
@@ -5071,7 +5277,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5082,7 +5288,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5096,22 +5302,22 @@
         <v>6</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>4</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5132,10 +5338,10 @@
         <v>9</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5156,10 +5362,10 @@
         <v>35</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5180,10 +5386,10 @@
         <v>62</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5204,10 +5410,10 @@
         <v>62</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -5256,7 +5462,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -5271,7 +5477,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5284,7 +5490,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5297,48 +5503,48 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>15</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>9</v>
@@ -5355,19 +5561,19 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>90</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>88</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>9</v>
@@ -5384,19 +5590,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>9</v>
@@ -5413,19 +5619,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>9</v>
@@ -5442,19 +5648,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>9</v>
@@ -5471,19 +5677,19 @@
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>9</v>
@@ -5500,19 +5706,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>15</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>9</v>
@@ -5529,19 +5735,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>14</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>9</v>
@@ -5558,19 +5764,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>9</v>
@@ -5587,19 +5793,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>8</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>9</v>
@@ -5616,19 +5822,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B14" s="4" t="n">
         <v>10</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>9</v>
@@ -5645,19 +5851,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>11</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>9</v>
@@ -5674,19 +5880,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>12</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>9</v>
@@ -5703,19 +5909,19 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>15</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>9</v>
@@ -5732,19 +5938,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B18" s="4" t="n">
         <v>18</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>9</v>
@@ -5761,19 +5967,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B19" s="4" t="n">
         <v>20</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>9</v>
@@ -5790,19 +5996,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B20" s="4" t="n">
         <v>19</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>9</v>
@@ -5819,19 +6025,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B21" s="4" t="n">
         <v>19</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>9</v>
@@ -5848,19 +6054,19 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B22" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>9</v>
@@ -5877,19 +6083,19 @@
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B23" s="4" t="n">
         <v>23</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>9</v>
@@ -5906,19 +6112,19 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B24" s="4" t="n">
         <v>13</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>9</v>
@@ -5935,19 +6141,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B25" s="4" t="n">
         <v>11</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>9</v>
@@ -5964,19 +6170,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B26" s="4" t="n">
         <v>9</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>9</v>
@@ -5993,19 +6199,19 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B27" s="4" t="n">
         <v>22</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>9</v>
@@ -6022,19 +6228,19 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B28" s="4" t="n">
         <v>16</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F28" s="4" t="s">
         <v>9</v>
@@ -6051,19 +6257,19 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B29" s="4" t="n">
         <v>17</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>9</v>
@@ -6080,19 +6286,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B30" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F30" s="4" t="s">
         <v>9</v>
@@ -6109,19 +6315,19 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B31" s="4" t="n">
         <v>18</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>9</v>
@@ -6138,19 +6344,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B32" s="4" t="n">
         <v>11</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>9</v>
@@ -6167,19 +6373,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B33" s="4" t="n">
         <v>24</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F33" s="4" t="s">
         <v>9</v>
@@ -6196,19 +6402,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B34" s="4" t="n">
         <v>25</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>9</v>
@@ -6225,19 +6431,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B35" s="4" t="n">
         <v>14</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F35" s="4" t="s">
         <v>35</v>
@@ -6252,19 +6458,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B36" s="4" t="n">
         <v>24</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>35</v>
@@ -6279,22 +6485,22 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B37" s="4" t="n">
         <v>25</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>6</v>
@@ -6302,23 +6508,25 @@
       <c r="H37" s="6" t="n">
         <v>46302</v>
       </c>
-      <c r="I37" s="4"/>
+      <c r="I37" s="6" t="n">
+        <v>46308</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B38" s="4" t="n">
         <v>14</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>62</v>
@@ -6331,19 +6539,19 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B39" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>9</v>
@@ -6360,19 +6568,19 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B40" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>9</v>
@@ -6389,19 +6597,19 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B41" s="4" t="n">
         <v>20</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F41" s="4" t="s">
         <v>9</v>
@@ -6418,19 +6626,19 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B42" s="4" t="n">
         <v>25</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>9</v>
@@ -6445,31 +6653,234 @@
         <v>46308</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F44" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="G44" s="8" t="n">
-        <f aca="false">SUM(G4:G42)</f>
+    <row r="43" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B43" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H43" s="6" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I43" s="6" t="n">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B44" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H44" s="6" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I44" s="6" t="n">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="5" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F45" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="G45" s="8" t="str">
-        <f aca="false">COUNTIF(F4:F42,"Terminado")&amp;" de "&amp;COUNTA(A4:A42)</f>
-        <v>35 de 39</v>
+      <c r="D45" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H45" s="6" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I45" s="6" t="n">
+        <v>46310</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F46" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="G46" s="9" t="n">
-        <f aca="false">SUMIF(F4:F42,"Terminado",G4:G42)/G44</f>
-        <v>0.912790697674419</v>
+      <c r="A46" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B46" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H46" s="6" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I46" s="6" t="n">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B47" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H47" s="6" t="n">
+        <v>46310</v>
+      </c>
+      <c r="I47" s="6" t="n">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B48" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G48" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H48" s="6" t="n">
+        <v>46315</v>
+      </c>
+      <c r="I48" s="6" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B49" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H49" s="6" t="n">
+        <v>46315</v>
+      </c>
+      <c r="I49" s="6" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F51" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="G51" s="8" t="n">
+        <f aca="false">SUM(G4:G49)</f>
+        <v>187</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F52" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="G52" s="8" t="str">
+        <f aca="false">COUNTIF(F4:F49,"Terminado")&amp;" de "&amp;COUNTA(A4:A49)</f>
+        <v>43 de 46</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F53" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="G53" s="9" t="n">
+        <f aca="false">SUMIF(F4:F49,"Terminado",G4:G49)/G51</f>
+        <v>0.951871657754011</v>
       </c>
     </row>
   </sheetData>
@@ -6477,7 +6888,7 @@
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F4:F42">
+  <conditionalFormatting sqref="F4:F49">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminado"</formula>
     </cfRule>
@@ -6504,7 +6915,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F4:F42" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F4:F49" type="list">
       <formula1>"Terminado,En desarrollo,Planeado"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -6524,7 +6935,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -6533,7 +6944,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6541,7 +6952,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6549,16 +6960,16 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>172</v>
+        <v>188</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6566,13 +6977,13 @@
         <v>46284</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6580,13 +6991,13 @@
         <v>46295</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>177</v>
+        <v>193</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>178</v>
+        <v>194</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>179</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6594,13 +7005,13 @@
         <v>46299</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>180</v>
+        <v>196</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>181</v>
+        <v>197</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6608,13 +7019,13 @@
         <v>46300</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>183</v>
+        <v>199</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>184</v>
+        <v>200</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>185</v>
+        <v>201</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6622,13 +7033,13 @@
         <v>46302</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>188</v>
+        <v>204</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6636,13 +7047,41 @@
         <v>46308</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>189</v>
+        <v>205</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>191</v>
+        <v>207</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>213</v>
       </c>
     </row>
   </sheetData>
@@ -6675,14 +7114,14 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>193</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6690,10 +7129,10 @@
         <v>4</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>195</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6701,12 +7140,12 @@
         <v>9</v>
       </c>
       <c r="B4" s="13" t="n">
-        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$29,A4)</f>
-        <v>22</v>
+        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$30,A4)</f>
+        <v>24</v>
       </c>
       <c r="C4" s="14" t="n">
         <f aca="false">IF(SUM($B$4:$B$7)=0,0,B4/SUM($B$4:$B$7))</f>
-        <v>0.846153846153846</v>
+        <v>0.888888888888889</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6714,12 +7153,12 @@
         <v>35</v>
       </c>
       <c r="B5" s="13" t="n">
-        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$29,A5)</f>
-        <v>3</v>
+        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$30,A5)</f>
+        <v>2</v>
       </c>
       <c r="C5" s="14" t="n">
         <f aca="false">IF(SUM($B$4:$B$7)=0,0,B5/SUM($B$4:$B$7))</f>
-        <v>0.115384615384615</v>
+        <v>0.0740740740740741</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6727,20 +7166,20 @@
         <v>62</v>
       </c>
       <c r="B6" s="13" t="n">
-        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$29,A6)</f>
+        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$30,A6)</f>
         <v>1</v>
       </c>
       <c r="C6" s="14" t="n">
         <f aca="false">IF(SUM($B$4:$B$7)=0,0,B6/SUM($B$4:$B$7))</f>
-        <v>0.0384615384615385</v>
+        <v>0.037037037037037</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>196</v>
+        <v>218</v>
       </c>
       <c r="B7" s="13" t="n">
-        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$29,A7)</f>
+        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$30,A7)</f>
         <v>0</v>
       </c>
       <c r="C7" s="14" t="n">
@@ -6750,11 +7189,11 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>197</v>
+        <v>219</v>
       </c>
       <c r="B8" s="15" t="n">
         <f aca="false">SUM(B4:B7)</f>
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -6777,7 +7216,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -6788,7 +7227,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>198</v>
+        <v>220</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6796,7 +7235,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>199</v>
+        <v>221</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6806,16 +7245,16 @@
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>200</v>
+        <v>222</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>201</v>
+        <v>223</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>202</v>
+        <v>224</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6823,16 +7262,16 @@
         <v>46284</v>
       </c>
       <c r="B4" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A4)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>172</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A4)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>187</v>
       </c>
       <c r="C4" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A4)</f>
-        <v>172</v>
+        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A4)</f>
+        <v>187</v>
       </c>
       <c r="D4" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A4)</f>
-        <v>39</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A4)</f>
+        <v>46</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6840,16 +7279,16 @@
         <v>46288</v>
       </c>
       <c r="B5" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A5)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>155.2</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A5)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>168.8</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A5)</f>
-        <v>172</v>
+        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A5)</f>
+        <v>187</v>
       </c>
       <c r="D5" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A5)</f>
-        <v>39</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A5)</f>
+        <v>46</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6857,16 +7296,16 @@
         <v>46291</v>
       </c>
       <c r="B6" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A6)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>142.6</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A6)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>155.1</v>
       </c>
       <c r="C6" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A6)</f>
-        <v>172</v>
+        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A6)</f>
+        <v>187</v>
       </c>
       <c r="D6" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A6)</f>
-        <v>39</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A6)</f>
+        <v>46</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6874,16 +7313,16 @@
         <v>46295</v>
       </c>
       <c r="B7" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A7)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>125.9</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A7)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>136.8</v>
       </c>
       <c r="C7" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A7)</f>
-        <v>134</v>
+        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A7)</f>
+        <v>149</v>
       </c>
       <c r="D7" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A7)</f>
-        <v>32</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A7)</f>
+        <v>39</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6891,16 +7330,16 @@
         <v>46299</v>
       </c>
       <c r="B8" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A8)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>109.1</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A8)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>118.6</v>
       </c>
       <c r="C8" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A8)</f>
-        <v>81</v>
+        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A8)</f>
+        <v>96</v>
       </c>
       <c r="D8" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A8)</f>
-        <v>23</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A8)</f>
+        <v>30</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6908,16 +7347,16 @@
         <v>46300</v>
       </c>
       <c r="B9" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A9)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>104.9</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A9)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>114</v>
       </c>
       <c r="C9" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A9)</f>
-        <v>31</v>
+        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A9)</f>
+        <v>46</v>
       </c>
       <c r="D9" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A9)</f>
-        <v>11</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A9)</f>
+        <v>18</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6925,16 +7364,16 @@
         <v>46302</v>
       </c>
       <c r="B10" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A10)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>96.5</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A10)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>104.9</v>
       </c>
       <c r="C10" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A10)</f>
-        <v>22</v>
+        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A10)</f>
+        <v>37</v>
       </c>
       <c r="D10" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A10)</f>
-        <v>7</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A10)</f>
+        <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6942,50 +7381,73 @@
         <v>46308</v>
       </c>
       <c r="B11" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A11)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>71.3</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A11)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>77.5</v>
       </c>
       <c r="C11" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$44-SUMIFS('Sprint Backlog'!$G$4:$G$42,'Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A11)</f>
-        <v>15</v>
+        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A11)</f>
+        <v>24</v>
       </c>
       <c r="D11" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-COUNTIFS('Sprint Backlog'!$F$4:$F$42,"Terminado",'Sprint Backlog'!$I$4:$I$42,"&lt;="&amp;A11)</f>
-        <v>4</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A11)</f>
+        <v>10</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="n">
-        <v>46316</v>
+        <v>46310</v>
       </c>
       <c r="B12" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A12)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>37.8</v>
-      </c>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
+        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A12)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>68.4</v>
+      </c>
+      <c r="C12" s="13" t="n">
+        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A12)</f>
+        <v>13</v>
+      </c>
+      <c r="D12" s="13" t="n">
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A12)</f>
+        <v>5</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="n">
-        <v>46323</v>
+        <v>46315</v>
       </c>
       <c r="B13" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A13)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>8.4</v>
-      </c>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
+        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A13)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>45.6</v>
+      </c>
+      <c r="C13" s="13" t="n">
+        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A13)</f>
+        <v>9</v>
+      </c>
+      <c r="D13" s="13" t="n">
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A13)</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="n">
-        <v>46325</v>
+        <v>46320</v>
       </c>
       <c r="B14" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$44*('Sprint Plan'!$D$5-A14)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>0</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A14)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>22.8</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="17" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B15" s="13" t="n">
+        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A15)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>0</v>
+      </c>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -7008,7 +7470,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -7018,25 +7480,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>204</v>
+        <v>226</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>202</v>
+        <v>224</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>205</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7046,10 +7508,10 @@
       </c>
       <c r="B4" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D4</f>
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="C4" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B4</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B4</f>
         <v>0</v>
       </c>
     </row>
@@ -7060,10 +7522,10 @@
       </c>
       <c r="B5" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D5</f>
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B5</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B5</f>
         <v>0</v>
       </c>
     </row>
@@ -7074,10 +7536,10 @@
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D6</f>
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="C6" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B6</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B6</f>
         <v>0</v>
       </c>
     </row>
@@ -7088,10 +7550,10 @@
       </c>
       <c r="B7" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D7</f>
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="C7" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B7</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B7</f>
         <v>7</v>
       </c>
     </row>
@@ -7102,10 +7564,10 @@
       </c>
       <c r="B8" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D8</f>
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C8" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B8</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B8</f>
         <v>16</v>
       </c>
     </row>
@@ -7116,10 +7578,10 @@
       </c>
       <c r="B9" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D9</f>
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C9" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B9</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B9</f>
         <v>28</v>
       </c>
     </row>
@@ -7130,10 +7592,10 @@
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D10</f>
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C10" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B10</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B10</f>
         <v>32</v>
       </c>
     </row>
@@ -7144,11 +7606,39 @@
       </c>
       <c r="B11" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D11</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C11" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$42)-B11</f>
-        <v>35</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B11</f>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="17" t="n">
+        <f aca="false">'Burn-down Chart'!A12</f>
+        <v>46310</v>
+      </c>
+      <c r="B12" s="13" t="n">
+        <f aca="false">'Burn-down Chart'!D12</f>
+        <v>5</v>
+      </c>
+      <c r="C12" s="13" t="n">
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B12</f>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="17" t="n">
+        <f aca="false">'Burn-down Chart'!A13</f>
+        <v>46315</v>
+      </c>
+      <c r="B13" s="13" t="n">
+        <f aca="false">'Burn-down Chart'!D13</f>
+        <v>3</v>
+      </c>
+      <c r="C13" s="13" t="n">
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B13</f>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -7171,7 +7661,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -7186,7 +7676,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>206</v>
+        <v>228</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7198,7 +7688,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>207</v>
+        <v>229</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7210,16 +7700,16 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>208</v>
+        <v>230</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>209</v>
+        <v>231</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>210</v>
+        <v>232</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>211</v>
+        <v>233</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>4</v>
@@ -7228,27 +7718,27 @@
         <v>2</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>212</v>
+        <v>234</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>213</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>214</v>
+        <v>236</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>215</v>
+        <v>237</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>216</v>
+        <v>238</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>15</v>
@@ -7257,24 +7747,24 @@
         <v>46299</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>218</v>
+        <v>240</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>219</v>
+        <v>241</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>220</v>
+        <v>242</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>221</v>
+        <v>243</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>14</v>
@@ -7283,24 +7773,24 @@
         <v>46300</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>222</v>
+        <v>244</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>223</v>
+        <v>245</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>224</v>
+        <v>246</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>225</v>
+        <v>247</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>19</v>
@@ -7309,24 +7799,24 @@
         <v>46300</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>226</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>227</v>
+        <v>249</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>228</v>
+        <v>250</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>229</v>
+        <v>251</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>15</v>
@@ -7335,24 +7825,24 @@
         <v>46300</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>218</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>230</v>
+        <v>252</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>231</v>
+        <v>253</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>232</v>
+        <v>254</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>17</v>
@@ -7361,24 +7851,24 @@
         <v>46300</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>222</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>233</v>
+        <v>255</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>234</v>
+        <v>256</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>235</v>
+        <v>257</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>11</v>
@@ -7387,24 +7877,24 @@
         <v>46300</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>226</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>236</v>
+        <v>258</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>237</v>
+        <v>259</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>238</v>
+        <v>260</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>18</v>
@@ -7413,24 +7903,24 @@
         <v>46300</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>218</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>239</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>217</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>13</v>
@@ -7439,24 +7929,24 @@
         <v>46300</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>222</v>
+        <v>244</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>242</v>
+        <v>264</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>243</v>
+        <v>265</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>244</v>
+        <v>266</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>19</v>
@@ -7465,24 +7955,24 @@
         <v>46300</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>222</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>245</v>
+        <v>267</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>246</v>
+        <v>268</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>247</v>
+        <v>269</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="F13" s="4" t="n">
         <v>22</v>
@@ -7491,24 +7981,24 @@
         <v>46300</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>218</v>
+        <v>240</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>248</v>
+        <v>270</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>249</v>
+        <v>271</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>250</v>
+        <v>272</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>17</v>
@@ -7517,24 +8007,24 @@
         <v>46300</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>226</v>
+        <v>248</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>251</v>
+        <v>273</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>252</v>
+        <v>274</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>253</v>
+        <v>275</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>11</v>
@@ -7543,24 +8033,24 @@
         <v>46302</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>226</v>
+        <v>248</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>254</v>
+        <v>276</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>255</v>
+        <v>277</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>256</v>
+        <v>278</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="F16" s="4" t="n">
         <v>20</v>
@@ -7569,24 +8059,24 @@
         <v>46302</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>222</v>
+        <v>244</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>257</v>
+        <v>279</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>258</v>
+        <v>280</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>259</v>
+        <v>281</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>260</v>
+        <v>282</v>
       </c>
       <c r="F17" s="4" t="n">
         <v>21</v>
@@ -7595,24 +8085,24 @@
         <v>46302</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>218</v>
+        <v>240</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>261</v>
+        <v>283</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>262</v>
+        <v>284</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>263</v>
+        <v>285</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="F18" s="4" t="n">
         <v>1</v>
@@ -7621,16 +8111,94 @@
         <v>46308</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D20" s="8" t="s">
-        <v>264</v>
-      </c>
-      <c r="E20" s="8" t="str">
-        <f aca="false">COUNTIF(E4:E18,"Corregido")&amp;" de "&amp;COUNTA(A4:A18)</f>
-        <v>14 de 15</v>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D23" s="8" t="s">
+        <v>295</v>
+      </c>
+      <c r="E23" s="8" t="str">
+        <f aca="false">COUNTIF(E4:E21,"Corregido")&amp;" de "&amp;COUNTA(A4:A21)</f>
+        <v>17 de 18</v>
       </c>
     </row>
   </sheetData>
@@ -7638,7 +8206,7 @@
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E4:E18">
+  <conditionalFormatting sqref="E4:E21">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminado"</formula>
     </cfRule>
@@ -7679,7 +8247,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -7693,7 +8261,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>265</v>
+        <v>296</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7704,7 +8272,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>266</v>
+        <v>297</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7715,22 +8283,22 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>267</v>
+        <v>298</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>268</v>
+        <v>299</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>269</v>
+        <v>300</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>270</v>
+        <v>301</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>271</v>
+        <v>302</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>4</v>
@@ -7738,350 +8306,392 @@
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>272</v>
+        <v>303</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>273</v>
+        <v>304</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>274</v>
+        <v>305</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>275</v>
+        <v>306</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>276</v>
+        <v>307</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>277</v>
+        <v>308</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>278</v>
+        <v>309</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>279</v>
+        <v>310</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>280</v>
+        <v>311</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>281</v>
+        <v>312</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>282</v>
+        <v>313</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>277</v>
+        <v>308</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>283</v>
+        <v>314</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>284</v>
+        <v>315</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>285</v>
+        <v>316</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>286</v>
+        <v>317</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>282</v>
+        <v>313</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>277</v>
+        <v>308</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>287</v>
+        <v>318</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>20</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>288</v>
+        <v>319</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>289</v>
+        <v>320</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>290</v>
+        <v>321</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>282</v>
+        <v>313</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>277</v>
+        <v>308</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>291</v>
+        <v>322</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>19</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>292</v>
+        <v>323</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>293</v>
+        <v>324</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>294</v>
+        <v>325</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>295</v>
+        <v>326</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>277</v>
+        <v>308</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>296</v>
+        <v>327</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>17</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>297</v>
+        <v>328</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>298</v>
+        <v>329</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>299</v>
+        <v>330</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>300</v>
+        <v>331</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>277</v>
+        <v>308</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>301</v>
+        <v>332</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>13</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>302</v>
+        <v>333</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>303</v>
+        <v>334</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>304</v>
+        <v>335</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>305</v>
+        <v>336</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>277</v>
+        <v>308</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>306</v>
+        <v>337</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>16</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>307</v>
+        <v>338</v>
       </c>
       <c r="D11" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>308</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>310</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>311</v>
+        <v>342</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>312</v>
+        <v>343</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>313</v>
+        <v>344</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>314</v>
+        <v>345</v>
       </c>
       <c r="F12" s="5"/>
       <c r="G12" s="4" t="s">
-        <v>315</v>
+        <v>346</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>316</v>
+        <v>347</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>317</v>
+        <v>348</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>318</v>
+        <v>349</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>319</v>
+        <v>350</v>
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="4" t="s">
-        <v>315</v>
+        <v>346</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>320</v>
+        <v>351</v>
       </c>
       <c r="B14" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>321</v>
+        <v>352</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>322</v>
+        <v>353</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>323</v>
+        <v>354</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>324</v>
+        <v>355</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>315</v>
+        <v>346</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>325</v>
+        <v>356</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>11</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>326</v>
+        <v>357</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>327</v>
+        <v>358</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>328</v>
+        <v>359</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>329</v>
+        <v>360</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>277</v>
+        <v>308</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>330</v>
+        <v>361</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>23</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>331</v>
+        <v>362</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>332</v>
+        <v>363</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>333</v>
+        <v>364</v>
       </c>
       <c r="F16" s="5"/>
       <c r="G16" s="4" t="s">
-        <v>315</v>
+        <v>346</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>334</v>
+        <v>365</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>24</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>335</v>
+        <v>366</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>336</v>
+        <v>367</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>337</v>
+        <v>368</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>338</v>
+        <v>369</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>315</v>
+        <v>346</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>339</v>
+        <v>370</v>
       </c>
       <c r="B18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>340</v>
+        <v>371</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>341</v>
+        <v>372</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>342</v>
+        <v>373</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>343</v>
+        <v>374</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F20" s="8" t="s">
-        <v>344</v>
-      </c>
-      <c r="G20" s="8" t="str">
-        <f aca="false">COUNTIF(G4:G18,"Aprobada")&amp;" de "&amp;COUNTA(A4:A18)</f>
-        <v>10 de 15</v>
+        <v>308</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="F19" s="5"/>
+      <c r="G19" s="4" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="F20" s="5"/>
+      <c r="G20" s="4" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F22" s="8" t="s">
+        <v>383</v>
+      </c>
+      <c r="G22" s="8" t="str">
+        <f aca="false">COUNTIF(G4:G20,"Aprobada")&amp;" de "&amp;COUNTA(A4:A20)</f>
+        <v>10 de 17</v>
       </c>
     </row>
   </sheetData>
@@ -8089,7 +8699,7 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G4:G18">
+  <conditionalFormatting sqref="G4:G20">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminado"</formula>
     </cfRule>
@@ -8119,7 +8729,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G4:G18" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G4:G20" type="list">
       <formula1>"Aprobada,Fallida,Pendiente"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Fondos con más capas en cada ala, ejecutable actualizado y notas para explicar el juego
</commit_message>
<xml_diff>
--- a/Documentacion/Producto2/PérezAlcántaraAlejandro_producción_10D_Sprint2.xlsx
+++ b/Documentacion/Producto2/PérezAlcántaraAlejandro_producción_10D_Sprint2.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="513">
   <si>
     <t xml:space="preserve">FEATURE LOG - ECOS DEL GRIMORIO (actualizado al Sprint 2)</t>
   </si>
@@ -576,6 +576,18 @@
     <t xml:space="preserve">Compilar la versión 1.0 del .exe y actualizar el manual</t>
   </si>
   <si>
+    <t xml:space="preserve">T47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fondos con más capas en cada ala (niebla, rayos de luz, estandartes, aves, aurora, libros y velas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guía para explicar cómo hice el juego y .exe con los fondos nuevos</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total horas:</t>
   </si>
   <si>
@@ -675,6 +687,15 @@
     <t xml:space="preserve">Ninguno.</t>
   </si>
   <si>
+    <t xml:space="preserve">Saltar nivel, versión 1.0 del .exe y documentos del Sprint 3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Darle más vida a los fondos de cada ala, compilar el .exe con los fondos nuevos y preparar mis notas para explicar el juego.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La primera compilación falló por falta de memoria; se volvió a compilar.</t>
+  </si>
+  <si>
     <t xml:space="preserve">PROJECT CHART - Estado general del proyecto</t>
   </si>
   <si>
@@ -1398,7 +1419,7 @@
     <t xml:space="preserve">T40, T43, T45</t>
   </si>
   <si>
-    <t xml:space="preserve">SPRINT REVIEW - SPRINT 2 (avance al 20 de octubre de 2026)</t>
+    <t xml:space="preserve">SPRINT REVIEW - SPRINT 2 (avance al 21 de octubre de 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Meta del sprint</t>
@@ -2347,7 +2368,7 @@
                   <c:v>15/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>20/10</c:v>
+                  <c:v>21/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>25/10</c:v>
@@ -2365,37 +2386,37 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>187</c:v>
+                  <c:v>192</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>168.8</c:v>
+                  <c:v>173.3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>155.1</c:v>
+                  <c:v>159.2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>136.8</c:v>
+                  <c:v>140.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>118.6</c:v>
+                  <c:v>121.8</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>114</c:v>
+                  <c:v>117.1</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>104.9</c:v>
+                  <c:v>107.7</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>77.5</c:v>
+                  <c:v>79.6</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>68.4</c:v>
+                  <c:v>70.2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>45.6</c:v>
+                  <c:v>42.1</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>22.8</c:v>
+                  <c:v>23.4</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -2491,7 +2512,7 @@
                   <c:v>15/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>20/10</c:v>
+                  <c:v>21/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>25/10</c:v>
@@ -2509,31 +2530,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>187</c:v>
+                  <c:v>192</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>187</c:v>
+                  <c:v>192</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>187</c:v>
+                  <c:v>192</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>149</c:v>
+                  <c:v>154</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>96</c:v>
+                  <c:v>101</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>46</c:v>
+                  <c:v>51</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>37</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>24</c:v>
+                  <c:v>29</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>13</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>9</c:v>
@@ -2551,11 +2572,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="26128128"/>
-        <c:axId val="12110244"/>
+        <c:axId val="28037859"/>
+        <c:axId val="98249806"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="26128128"/>
+        <c:axId val="28037859"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2621,7 +2642,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12110244"/>
+        <c:crossAx val="98249806"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2629,7 +2650,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="12110244"/>
+        <c:axId val="98249806"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2705,7 +2726,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26128128"/>
+        <c:crossAx val="28037859"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2887,7 +2908,7 @@
                   <c:v>15/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>20/10</c:v>
+                  <c:v>21/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2899,31 +2920,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>46</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>46</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>46</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>39</c:v>
+                  <c:v>41</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>30</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>18</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>14</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>10</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>5</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>3</c:v>
@@ -3019,7 +3040,7 @@
                   <c:v>15/10</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>20/10</c:v>
+                  <c:v>21/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3058,7 +3079,7 @@
                   <c:v>41</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>43</c:v>
+                  <c:v>45</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3073,11 +3094,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="15060964"/>
-        <c:axId val="64371788"/>
+        <c:axId val="10223766"/>
+        <c:axId val="63904845"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="15060964"/>
+        <c:axId val="10223766"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3143,7 +3164,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64371788"/>
+        <c:crossAx val="63904845"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3151,7 +3172,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="64371788"/>
+        <c:axId val="63904845"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3227,7 +3248,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15060964"/>
+        <c:crossAx val="10223766"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4219,7 +4240,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4228,7 +4249,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4237,16 +4258,16 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>4</v>
@@ -4254,13 +4275,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>141</v>
@@ -4272,13 +4293,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>93</v>
@@ -4290,13 +4311,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>119</v>
@@ -4308,13 +4329,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>101</v>
@@ -4326,16 +4347,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="E8" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C8,FIND(",",C8&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
@@ -4344,13 +4365,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>137</v>
@@ -4362,16 +4383,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="E10" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C10,FIND(",",C10&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
@@ -4380,16 +4401,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="E11" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C11,FIND(",",C11&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
@@ -4398,13 +4419,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>127</v>
@@ -4416,16 +4437,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="E13" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C13,FIND(",",C13&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
@@ -4434,16 +4455,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="E14" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C14,FIND(",",C14&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
@@ -4452,13 +4473,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>135</v>
@@ -4470,16 +4491,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="E16" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C16,FIND(",",C16&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
@@ -4488,16 +4509,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="E17" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C17,FIND(",",C17&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
@@ -4506,13 +4527,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>113</v>
@@ -4524,13 +4545,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>129</v>
@@ -4542,16 +4563,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>442</v>
+        <v>449</v>
       </c>
       <c r="E20" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C20,FIND(",",C20&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
@@ -4560,16 +4581,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>444</v>
+        <v>451</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="E21" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C21,FIND(",",C21&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
@@ -4578,16 +4599,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
       <c r="E22" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C22,FIND(",",C22&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
@@ -4596,16 +4617,16 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="E23" s="4" t="str">
         <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C23,FIND(",",C23&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
@@ -4667,39 +4688,39 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>456</v>
+        <v>463</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
       <c r="B4" s="5" t="str">
-        <f aca="false">COUNTIF('Sprint Backlog'!$F$4:$F$49,"Terminado")&amp;" de "&amp;COUNTA('Sprint Backlog'!$A$4:$A$49)</f>
-        <v>43 de 46</v>
+        <f aca="false">COUNTIF('Sprint Backlog'!$F$4:$F$51,"Terminado")&amp;" de "&amp;COUNTA('Sprint Backlog'!$A$4:$A$51)</f>
+        <v>45 de 48</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>459</v>
+        <v>466</v>
       </c>
       <c r="B5" s="5" t="str">
-        <f aca="false">SUMIF('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$G$4:$G$49)&amp;" de "&amp;'Sprint Backlog'!$G$51&amp;" hrs"</f>
-        <v>178 de 187 hrs</v>
+        <f aca="false">SUMIF('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$G$4:$G$51)&amp;" de "&amp;'Sprint Backlog'!$G$53&amp;" hrs"</f>
+        <v>183 de 192 hrs</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>460</v>
+        <v>467</v>
       </c>
       <c r="B6" s="5" t="str">
         <f aca="false">COUNTIF('Feature Log'!$C$4:$C$30,"Terminado")&amp;" de "&amp;COUNTA('Feature Log'!$A$4:$A$30)</f>
@@ -4708,7 +4729,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
       <c r="B7" s="5" t="str">
         <f aca="false">COUNTIF(Buglist!$E$4:$E$21,"Corregido")&amp;" de "&amp;COUNTA(Buglist!$A$4:$A$21)</f>
@@ -4717,7 +4738,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="B8" s="5" t="str">
         <f aca="false">COUNTIF('Pruebas Alfa'!$G$4:$G$20,"Aprobada")&amp;" de "&amp;COUNTA('Pruebas Alfa'!$A$4:$A$20)</f>
@@ -4726,42 +4747,42 @@
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>463</v>
+        <v>470</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>464</v>
+        <v>471</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>465</v>
+        <v>472</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>466</v>
+        <v>473</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>467</v>
+        <v>474</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>468</v>
+        <v>475</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>469</v>
+        <v>476</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>472</v>
+        <v>479</v>
       </c>
     </row>
   </sheetData>
@@ -4802,7 +4823,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>473</v>
+        <v>480</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4820,7 +4841,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>474</v>
+        <v>481</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4838,43 +4859,43 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>475</v>
+        <v>482</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>476</v>
+        <v>483</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>477</v>
+        <v>484</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>479</v>
+        <v>486</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>480</v>
+        <v>487</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>481</v>
+        <v>488</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>482</v>
+        <v>489</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>483</v>
+        <v>490</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>484</v>
+        <v>491</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>485</v>
+        <v>492</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>4</v>
@@ -4882,7 +4903,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>486</v>
+        <v>493</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="5"/>
@@ -4900,7 +4921,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>487</v>
+        <v>494</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="5"/>
@@ -4918,7 +4939,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>488</v>
+        <v>495</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="5"/>
@@ -4936,7 +4957,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>489</v>
+        <v>496</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="5"/>
@@ -4954,7 +4975,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>490</v>
+        <v>497</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="5"/>
@@ -4972,7 +4993,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>491</v>
+        <v>498</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="5"/>
@@ -4990,7 +5011,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>492</v>
+        <v>499</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="5"/>
@@ -5008,7 +5029,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>493</v>
+        <v>500</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="5"/>
@@ -5026,7 +5047,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>494</v>
+        <v>501</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="5"/>
@@ -5044,7 +5065,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>495</v>
+        <v>502</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="5"/>
@@ -5062,7 +5083,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>496</v>
+        <v>503</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="5"/>
@@ -5080,7 +5101,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>497</v>
+        <v>504</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="5"/>
@@ -5098,7 +5119,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>498</v>
+        <v>505</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="5"/>
@@ -5116,7 +5137,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>499</v>
+        <v>506</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="5"/>
@@ -5134,7 +5155,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>500</v>
+        <v>507</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="5"/>
@@ -5152,7 +5173,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F20" s="8" t="s">
-        <v>501</v>
+        <v>508</v>
       </c>
       <c r="H20" s="19" t="n">
         <f aca="false">COUNTA(C4:C18)</f>
@@ -5161,7 +5182,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F21" s="8" t="s">
-        <v>502</v>
+        <v>509</v>
       </c>
       <c r="H21" s="0" t="str">
         <f aca="false">IF(COUNT(H4:H18)=0,"",ROUND(AVERAGE(H4:H18),1))</f>
@@ -5170,7 +5191,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F22" s="8" t="s">
-        <v>503</v>
+        <v>510</v>
       </c>
       <c r="H22" s="0" t="str">
         <f aca="false">IF(COUNT(I4:I18)=0,"",ROUND(AVERAGE(I4:I18),1))</f>
@@ -5179,7 +5200,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F23" s="8" t="s">
-        <v>504</v>
+        <v>511</v>
       </c>
       <c r="H23" s="0" t="str">
         <f aca="false">IF(COUNT(J4:J18)=0,"",ROUND(AVERAGE(J4:J18),1))</f>
@@ -5188,7 +5209,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F24" s="8" t="s">
-        <v>505</v>
+        <v>512</v>
       </c>
       <c r="H24" s="19" t="n">
         <f aca="false">COUNTIF(F4:F18,"Terminó el juego")</f>
@@ -5462,7 +5483,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -6856,31 +6877,89 @@
         <v>46315</v>
       </c>
     </row>
+    <row r="50" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B50" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H50" s="6" t="n">
+        <v>46316</v>
+      </c>
+      <c r="I50" s="6" t="n">
+        <v>46316</v>
+      </c>
+    </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F51" s="8" t="s">
-        <v>181</v>
-      </c>
-      <c r="G51" s="8" t="n">
-        <f aca="false">SUM(G4:G49)</f>
-        <v>187</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F52" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="G52" s="8" t="str">
-        <f aca="false">COUNTIF(F4:F49,"Terminado")&amp;" de "&amp;COUNTA(A4:A49)</f>
-        <v>43 de 46</v>
+      <c r="A51" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B51" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E51" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G51" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H51" s="6" t="n">
+        <v>46316</v>
+      </c>
+      <c r="I51" s="6" t="n">
+        <v>46316</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F53" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="G53" s="9" t="n">
-        <f aca="false">SUMIF(F4:F49,"Terminado",G4:G49)/G51</f>
-        <v>0.951871657754011</v>
+        <v>185</v>
+      </c>
+      <c r="G53" s="8" t="n">
+        <f aca="false">SUM(G4:G51)</f>
+        <v>192</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F54" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="G54" s="8" t="str">
+        <f aca="false">COUNTIF(F4:F51,"Terminado")&amp;" de "&amp;COUNTA(A4:A51)</f>
+        <v>45 de 48</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F55" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="G55" s="9" t="n">
+        <f aca="false">SUMIF(F4:F51,"Terminado",G4:G51)/G53</f>
+        <v>0.953125</v>
       </c>
     </row>
   </sheetData>
@@ -6888,7 +6967,7 @@
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F4:F49">
+  <conditionalFormatting sqref="F4:F51">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminado"</formula>
     </cfRule>
@@ -6915,7 +6994,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F4:F49" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F4:F51" type="list">
       <formula1>"Terminado,En desarrollo,Planeado"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -6935,7 +7014,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -6944,7 +7023,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6952,7 +7031,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -6960,16 +7039,16 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6977,13 +7056,13 @@
         <v>46284</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6991,13 +7070,13 @@
         <v>46295</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7005,13 +7084,13 @@
         <v>46299</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7019,13 +7098,13 @@
         <v>46300</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7033,13 +7112,13 @@
         <v>46302</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7047,13 +7126,13 @@
         <v>46308</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7061,13 +7140,13 @@
         <v>46310</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7075,13 +7154,27 @@
         <v>46315</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>213</v>
+        <v>217</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -7114,14 +7207,14 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7129,10 +7222,10 @@
         <v>4</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7176,7 +7269,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="B7" s="13" t="n">
         <f aca="false">COUNTIF('Feature Log'!$C$4:$C$30,A7)</f>
@@ -7189,7 +7282,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="B8" s="15" t="n">
         <f aca="false">SUM(B4:B7)</f>
@@ -7227,7 +7320,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7235,7 +7328,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7245,16 +7338,16 @@
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7262,16 +7355,16 @@
         <v>46284</v>
       </c>
       <c r="B4" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A4)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>187</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A4)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>192</v>
       </c>
       <c r="C4" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A4)</f>
-        <v>187</v>
+        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A4)</f>
+        <v>192</v>
       </c>
       <c r="D4" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A4)</f>
-        <v>46</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A4)</f>
+        <v>48</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7279,16 +7372,16 @@
         <v>46288</v>
       </c>
       <c r="B5" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A5)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>168.8</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A5)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>173.3</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A5)</f>
-        <v>187</v>
+        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A5)</f>
+        <v>192</v>
       </c>
       <c r="D5" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A5)</f>
-        <v>46</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A5)</f>
+        <v>48</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7296,16 +7389,16 @@
         <v>46291</v>
       </c>
       <c r="B6" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A6)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>155.1</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A6)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>159.2</v>
       </c>
       <c r="C6" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A6)</f>
-        <v>187</v>
+        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A6)</f>
+        <v>192</v>
       </c>
       <c r="D6" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A6)</f>
-        <v>46</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A6)</f>
+        <v>48</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7313,16 +7406,16 @@
         <v>46295</v>
       </c>
       <c r="B7" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A7)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>136.8</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A7)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>140.5</v>
       </c>
       <c r="C7" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A7)</f>
-        <v>149</v>
+        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A7)</f>
+        <v>154</v>
       </c>
       <c r="D7" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A7)</f>
-        <v>39</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A7)</f>
+        <v>41</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7330,16 +7423,16 @@
         <v>46299</v>
       </c>
       <c r="B8" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A8)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>118.6</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A8)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>121.8</v>
       </c>
       <c r="C8" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A8)</f>
-        <v>96</v>
+        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A8)</f>
+        <v>101</v>
       </c>
       <c r="D8" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A8)</f>
-        <v>30</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A8)</f>
+        <v>32</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7347,16 +7440,16 @@
         <v>46300</v>
       </c>
       <c r="B9" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A9)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>114</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A9)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>117.1</v>
       </c>
       <c r="C9" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A9)</f>
-        <v>46</v>
+        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A9)</f>
+        <v>51</v>
       </c>
       <c r="D9" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A9)</f>
-        <v>18</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A9)</f>
+        <v>20</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7364,16 +7457,16 @@
         <v>46302</v>
       </c>
       <c r="B10" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A10)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>104.9</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A10)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>107.7</v>
       </c>
       <c r="C10" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A10)</f>
-        <v>37</v>
+        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A10)</f>
+        <v>42</v>
       </c>
       <c r="D10" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A10)</f>
-        <v>14</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A10)</f>
+        <v>16</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7381,16 +7474,16 @@
         <v>46308</v>
       </c>
       <c r="B11" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A11)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>77.5</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A11)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>79.6</v>
       </c>
       <c r="C11" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A11)</f>
-        <v>24</v>
+        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A11)</f>
+        <v>29</v>
       </c>
       <c r="D11" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A11)</f>
-        <v>10</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A11)</f>
+        <v>12</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7398,32 +7491,32 @@
         <v>46310</v>
       </c>
       <c r="B12" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A12)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>68.4</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A12)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>70.2</v>
       </c>
       <c r="C12" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A12)</f>
-        <v>13</v>
+        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A12)</f>
+        <v>18</v>
       </c>
       <c r="D12" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A12)</f>
-        <v>5</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A12)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B13" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A13)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>45.6</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A13)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>42.1</v>
       </c>
       <c r="C13" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$51-SUMIFS('Sprint Backlog'!$G$4:$G$49,'Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A13)</f>
+        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A13)</f>
         <v>9</v>
       </c>
       <c r="D13" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-COUNTIFS('Sprint Backlog'!$F$4:$F$49,"Terminado",'Sprint Backlog'!$I$4:$I$49,"&lt;="&amp;A13)</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A13)</f>
         <v>3</v>
       </c>
     </row>
@@ -7432,8 +7525,8 @@
         <v>46320</v>
       </c>
       <c r="B14" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A14)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>22.8</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A14)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>23.4</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
@@ -7443,7 +7536,7 @@
         <v>46325</v>
       </c>
       <c r="B15" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$51*('Sprint Plan'!$D$5-A15)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A15)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
         <v>0</v>
       </c>
       <c r="C15" s="13"/>
@@ -7480,25 +7573,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7508,10 +7601,10 @@
       </c>
       <c r="B4" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D4</f>
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C4" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B4</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B4</f>
         <v>0</v>
       </c>
     </row>
@@ -7522,10 +7615,10 @@
       </c>
       <c r="B5" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D5</f>
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B5</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B5</f>
         <v>0</v>
       </c>
     </row>
@@ -7536,10 +7629,10 @@
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D6</f>
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C6" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B6</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B6</f>
         <v>0</v>
       </c>
     </row>
@@ -7550,10 +7643,10 @@
       </c>
       <c r="B7" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D7</f>
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C7" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B7</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B7</f>
         <v>7</v>
       </c>
     </row>
@@ -7564,10 +7657,10 @@
       </c>
       <c r="B8" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D8</f>
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C8" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B8</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B8</f>
         <v>16</v>
       </c>
     </row>
@@ -7578,10 +7671,10 @@
       </c>
       <c r="B9" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D9</f>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C9" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B9</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B9</f>
         <v>28</v>
       </c>
     </row>
@@ -7592,10 +7685,10 @@
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D10</f>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C10" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B10</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B10</f>
         <v>32</v>
       </c>
     </row>
@@ -7606,10 +7699,10 @@
       </c>
       <c r="B11" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D11</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C11" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B11</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B11</f>
         <v>36</v>
       </c>
     </row>
@@ -7620,25 +7713,25 @@
       </c>
       <c r="B12" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D12</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C12" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B12</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B12</f>
         <v>41</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="n">
         <f aca="false">'Burn-down Chart'!A13</f>
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B13" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D13</f>
         <v>3</v>
       </c>
       <c r="C13" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$49)-B13</f>
-        <v>43</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B13</f>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -7676,7 +7769,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7688,7 +7781,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7700,16 +7793,16 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>4</v>
@@ -7718,27 +7811,27 @@
         <v>2</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>15</v>
@@ -7747,24 +7840,24 @@
         <v>46299</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>14</v>
@@ -7773,24 +7866,24 @@
         <v>46300</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>19</v>
@@ -7799,24 +7892,24 @@
         <v>46300</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>15</v>
@@ -7825,24 +7918,24 @@
         <v>46300</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>17</v>
@@ -7851,24 +7944,24 @@
         <v>46300</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>11</v>
@@ -7877,24 +7970,24 @@
         <v>46300</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>18</v>
@@ -7903,24 +7996,24 @@
         <v>46300</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>13</v>
@@ -7929,24 +8022,24 @@
         <v>46300</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>19</v>
@@ -7955,24 +8048,24 @@
         <v>46300</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F13" s="4" t="n">
         <v>22</v>
@@ -7981,24 +8074,24 @@
         <v>46300</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>17</v>
@@ -8007,24 +8100,24 @@
         <v>46300</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>11</v>
@@ -8033,24 +8126,24 @@
         <v>46302</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F16" s="4" t="n">
         <v>20</v>
@@ -8059,24 +8152,24 @@
         <v>46302</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="F17" s="4" t="n">
         <v>21</v>
@@ -8085,24 +8178,24 @@
         <v>46302</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F18" s="4" t="n">
         <v>1</v>
@@ -8111,24 +8204,24 @@
         <v>46308</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F19" s="4" t="n">
         <v>10</v>
@@ -8137,24 +8230,24 @@
         <v>46310</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F20" s="4" t="n">
         <v>1</v>
@@ -8163,24 +8256,24 @@
         <v>46310</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>89</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="F21" s="4" t="n">
         <v>23</v>
@@ -8189,12 +8282,12 @@
         <v>46310</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D23" s="8" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="E23" s="8" t="str">
         <f aca="false">COUNTIF(E4:E21,"Corregido")&amp;" de "&amp;COUNTA(A4:A21)</f>
@@ -8261,7 +8354,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8272,7 +8365,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -8283,22 +8376,22 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>4</v>
@@ -8306,388 +8399,388 @@
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>323</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>320</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>315</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>316</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>317</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>313</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>20</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="D7" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>320</v>
       </c>
-      <c r="E7" s="5" t="s">
-        <v>321</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>313</v>
-      </c>
       <c r="G7" s="4" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>19</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>17</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>13</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>16</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="F12" s="5"/>
       <c r="G12" s="4" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="4" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="B14" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="D14" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>353</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>354</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>355</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>11</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>360</v>
+        <v>367</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>23</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="F16" s="5"/>
       <c r="G16" s="4" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>24</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>366</v>
+        <v>373</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>367</v>
+        <v>374</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>370</v>
+        <v>377</v>
       </c>
       <c r="B18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>371</v>
+        <v>378</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="B19" s="4" t="n">
         <v>27</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>376</v>
+        <v>383</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="F19" s="5"/>
       <c r="G19" s="4" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="B20" s="4" t="n">
         <v>27</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="F20" s="5"/>
       <c r="G20" s="4" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F22" s="8" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="G22" s="8" t="str">
         <f aca="false">COUNTIF(G4:G20,"Aprobada")&amp;" de "&amp;COUNTA(A4:A20)</f>

</xml_diff>

<commit_message>
Versión web para celular: controles táctiles, plantilla para instalarla como app y documentos actualizados
</commit_message>
<xml_diff>
--- a/Documentacion/Producto2/PérezAlcántaraAlejandro_producción_10D_Sprint2.xlsx
+++ b/Documentacion/Producto2/PérezAlcántaraAlejandro_producción_10D_Sprint2.xlsx
@@ -31,12 +31,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="522">
   <si>
     <t xml:space="preserve">FEATURE LOG - ECOS DEL GRIMORIO (actualizado al Sprint 2)</t>
   </si>
   <si>
-    <t xml:space="preserve">Los features 1 a 14 vienen del Feature Log inicial (GDD 3.1); del 15 al 26 se agregaron en el Sprint 2 para cubrir secciones del GDD que no tenían feature; el 27 salió de las pruebas.</t>
+    <t xml:space="preserve">Los features 1 a 14 vienen del Feature Log inicial (GDD 3.1); del 15 al 26 se agregaron en el Sprint 2 para cubrir secciones del GDD que no tenían feature; el 27 salió de las pruebas y el 28 de la revisión en clase.</t>
   </si>
   <si>
     <t xml:space="preserve">Featureid</t>
@@ -231,6 +231,12 @@
     <t xml:space="preserve">Agregado después de las pruebas del 14 y 15 de octubre y de la revisión en clase</t>
   </si>
   <si>
+    <t xml:space="preserve">Versión web para celular (WebGL + PWA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedido del profe en la revisión. Botones táctiles, plantilla para instalarlo como app y publicación en GitHub Pages</t>
+  </si>
+  <si>
     <t xml:space="preserve">SPRINT PLAN - ECOS DEL GRIMORIO (replaneado en el Sprint 2)</t>
   </si>
   <si>
@@ -588,6 +594,12 @@
     <t xml:space="preserve">Guía para explicar cómo hice el juego y .exe con los fondos nuevos</t>
   </si>
   <si>
+    <t xml:space="preserve">T49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Versión web para celular: botones táctiles, plantilla PWA y publicación en GitHub Pages</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total horas:</t>
   </si>
   <si>
@@ -696,6 +708,15 @@
     <t xml:space="preserve">La primera compilación falló por falta de memoria; se volvió a compilar.</t>
   </si>
   <si>
+    <t xml:space="preserve">Fondos nuevos en las cinco alas, .exe compilado otra vez y guía para explicar el juego.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Versión para celular que pidió el profe: botones táctiles, versión web que se instala como app y publicarla en GitHub Pages.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La primera compilación para web tarda porque Unity reimporta todo al cambiar de plataforma.</t>
+  </si>
+  <si>
     <t xml:space="preserve">PROJECT CHART - Estado general del proyecto</t>
   </si>
   <si>
@@ -1417,6 +1438,12 @@
   </si>
   <si>
     <t xml:space="preserve">T40, T43, T45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Versión web para celular (navegador y app)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28</t>
   </si>
   <si>
     <t xml:space="preserve">SPRINT REVIEW - SPRINT 2 (avance al 21 de octubre de 2026)</t>
@@ -2172,7 +2199,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>24</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>2</c:v>
@@ -2337,9 +2364,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Burn-down Chart'!$A$4:$A$15</c:f>
+              <c:f>'Burn-down Chart'!$A$4:$A$16</c:f>
               <c:strCache>
-                <c:ptCount val="12"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>19/09</c:v>
                 </c:pt>
@@ -2371,9 +2398,12 @@
                   <c:v>21/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>22/10</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>25/10</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="12">
                   <c:v>30/10</c:v>
                 </c:pt>
               </c:strCache>
@@ -2381,44 +2411,47 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Burn-down Chart'!$B$4:$B$15</c:f>
+              <c:f>'Burn-down Chart'!$B$4:$B$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>192</c:v>
+                  <c:v>198</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>173.3</c:v>
+                  <c:v>178.7</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>159.2</c:v>
+                  <c:v>164.2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>140.5</c:v>
+                  <c:v>144.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>121.8</c:v>
+                  <c:v>125.6</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>117.1</c:v>
+                  <c:v>120.7</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>107.7</c:v>
+                  <c:v>111.1</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>79.6</c:v>
+                  <c:v>82.1</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>70.2</c:v>
+                  <c:v>72.4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>42.1</c:v>
+                  <c:v>43.5</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>23.4</c:v>
+                  <c:v>38.6</c:v>
                 </c:pt>
                 <c:pt idx="11">
+                  <c:v>24.1</c:v>
+                </c:pt>
+                <c:pt idx="12">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -2481,9 +2514,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Burn-down Chart'!$A$4:$A$15</c:f>
+              <c:f>'Burn-down Chart'!$A$4:$A$16</c:f>
               <c:strCache>
-                <c:ptCount val="12"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>19/09</c:v>
                 </c:pt>
@@ -2515,9 +2548,12 @@
                   <c:v>21/10</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>22/10</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>25/10</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="12">
                   <c:v>30/10</c:v>
                 </c:pt>
               </c:strCache>
@@ -2525,38 +2561,41 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Burn-down Chart'!$C$4:$C$15</c:f>
+              <c:f>'Burn-down Chart'!$C$4:$C$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>192</c:v>
+                  <c:v>198</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>192</c:v>
+                  <c:v>198</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>192</c:v>
+                  <c:v>198</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>154</c:v>
+                  <c:v>160</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>101</c:v>
+                  <c:v>107</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>51</c:v>
+                  <c:v>57</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>42</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>29</c:v>
+                  <c:v>35</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>18</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="9">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>9</c:v>
                 </c:pt>
               </c:numCache>
@@ -2572,11 +2611,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="28037859"/>
-        <c:axId val="98249806"/>
+        <c:axId val="80088730"/>
+        <c:axId val="11949119"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="28037859"/>
+        <c:axId val="80088730"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2642,7 +2681,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98249806"/>
+        <c:crossAx val="11949119"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2650,7 +2689,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="98249806"/>
+        <c:axId val="11949119"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2726,7 +2765,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="28037859"/>
+        <c:crossAx val="80088730"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2877,9 +2916,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Task Chart'!$A$4:$A$13</c:f>
+              <c:f>'Task Chart'!$A$4:$A$14</c:f>
               <c:strCache>
-                <c:ptCount val="10"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
                   <c:v>19/09</c:v>
                 </c:pt>
@@ -2909,44 +2948,50 @@
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>21/10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>22/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Task Chart'!$B$4:$B$13</c:f>
+              <c:f>'Task Chart'!$B$4:$B$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>48</c:v>
+                  <c:v>49</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>48</c:v>
+                  <c:v>49</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>48</c:v>
+                  <c:v>49</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>41</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>32</c:v>
+                  <c:v>33</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>20</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>16</c:v>
+                  <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>12</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="9">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
@@ -3009,9 +3054,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Task Chart'!$A$4:$A$13</c:f>
+              <c:f>'Task Chart'!$A$4:$A$14</c:f>
               <c:strCache>
-                <c:ptCount val="10"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
                   <c:v>19/09</c:v>
                 </c:pt>
@@ -3041,16 +3086,19 @@
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>21/10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>22/10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Task Chart'!$C$4:$C$13</c:f>
+              <c:f>'Task Chart'!$C$4:$C$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -3080,6 +3128,9 @@
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>46</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3094,11 +3145,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="10223766"/>
-        <c:axId val="63904845"/>
+        <c:axId val="77556814"/>
+        <c:axId val="80734995"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="10223766"/>
+        <c:axId val="77556814"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3164,7 +3215,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63904845"/>
+        <c:crossAx val="80734995"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3172,7 +3223,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="63904845"/>
+        <c:axId val="80734995"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3248,7 +3299,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10223766"/>
+        <c:crossAx val="77556814"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3585,7 +3636,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -4176,12 +4227,32 @@
         <v>65</v>
       </c>
     </row>
+    <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
   </mergeCells>
-  <conditionalFormatting sqref="C4:C30">
+  <conditionalFormatting sqref="C4:C31">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminado"</formula>
     </cfRule>
@@ -4208,7 +4279,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C4:C30" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C4:C31" type="list">
       <formula1>"Terminado,En desarrollo,Planeado,Sin planear"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4228,7 +4299,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -4240,7 +4311,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4249,7 +4320,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4258,16 +4329,16 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>4</v>
@@ -4275,361 +4346,379 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E4" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C4,FIND(",",C4&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C4,FIND(",",C4&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E5" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C5,FIND(",",C5&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C5,FIND(",",C5&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E6" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C6,FIND(",",C6&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C6,FIND(",",C6&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E7" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C7,FIND(",",C7&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C7,FIND(",",C7&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="E8" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C8,FIND(",",C8&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C8,FIND(",",C8&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E9" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C9,FIND(",",C9&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C9,FIND(",",C9&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="E10" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C10,FIND(",",C10&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C10,FIND(",",C10&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="E11" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C11,FIND(",",C11&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C11,FIND(",",C11&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E12" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C12,FIND(",",C12&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C12,FIND(",",C12&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="E13" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C13,FIND(",",C13&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C13,FIND(",",C13&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="E14" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C14,FIND(",",C14&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C14,FIND(",",C14&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E15" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C15,FIND(",",C15&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C15,FIND(",",C15&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="E16" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C16,FIND(",",C16&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C16,FIND(",",C16&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
       <c r="E17" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C17,FIND(",",C17&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C17,FIND(",",C17&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>442</v>
+        <v>449</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E18" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C18,FIND(",",C18&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C18,FIND(",",C18&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>444</v>
+        <v>451</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E19" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C19,FIND(",",C19&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C19,FIND(",",C19&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="E20" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C20,FIND(",",C20&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C20,FIND(",",C20&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
       <c r="E21" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C21,FIND(",",C21&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C21,FIND(",",C21&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>En desarrollo</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>456</v>
+        <v>463</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="E22" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C22,FIND(",",C22&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C22,FIND(",",C22&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>En desarrollo</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>459</v>
+        <v>466</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>460</v>
+        <v>467</v>
       </c>
       <c r="D23" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="E23" s="4" t="str">
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C23,FIND(",",C23&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
+        <v>Terminado</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
         <v>461</v>
       </c>
-      <c r="E23" s="4" t="str">
-        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$30,MATCH(VALUE(LEFT(C23,FIND(",",C23&amp;",")-1)),'Feature Log'!$A$4:$A$30,0)),"")</f>
+      <c r="B24" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>470</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="E24" s="4" t="str">
+        <f aca="false">IFERROR(INDEX('Feature Log'!$C$4:$C$31,MATCH(VALUE(LEFT(C24,FIND(",",C24&amp;",")-1)),'Feature Log'!$A$4:$A$31,0)),"")</f>
         <v>Terminado</v>
       </c>
     </row>
@@ -4638,7 +4727,7 @@
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E4:E23">
+  <conditionalFormatting sqref="E4:E24">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminado"</formula>
     </cfRule>
@@ -4688,48 +4777,48 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>462</v>
+        <v>471</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>463</v>
+        <v>472</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>464</v>
+        <v>473</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>465</v>
+        <v>474</v>
       </c>
       <c r="B4" s="5" t="str">
-        <f aca="false">COUNTIF('Sprint Backlog'!$F$4:$F$51,"Terminado")&amp;" de "&amp;COUNTA('Sprint Backlog'!$A$4:$A$51)</f>
-        <v>45 de 48</v>
+        <f aca="false">COUNTIF('Sprint Backlog'!$F$4:$F$52,"Terminado")&amp;" de "&amp;COUNTA('Sprint Backlog'!$A$4:$A$52)</f>
+        <v>46 de 49</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>466</v>
+        <v>475</v>
       </c>
       <c r="B5" s="5" t="str">
-        <f aca="false">SUMIF('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$G$4:$G$51)&amp;" de "&amp;'Sprint Backlog'!$G$53&amp;" hrs"</f>
-        <v>183 de 192 hrs</v>
+        <f aca="false">SUMIF('Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$G$4:$G$52)&amp;" de "&amp;'Sprint Backlog'!$G$54&amp;" hrs"</f>
+        <v>189 de 198 hrs</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>467</v>
+        <v>476</v>
       </c>
       <c r="B6" s="5" t="str">
-        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$30,"Terminado")&amp;" de "&amp;COUNTA('Feature Log'!$A$4:$A$30)</f>
-        <v>24 de 27</v>
+        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$31,"Terminado")&amp;" de "&amp;COUNTA('Feature Log'!$A$4:$A$31)</f>
+        <v>25 de 28</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>468</v>
+        <v>477</v>
       </c>
       <c r="B7" s="5" t="str">
         <f aca="false">COUNTIF(Buglist!$E$4:$E$21,"Corregido")&amp;" de "&amp;COUNTA(Buglist!$A$4:$A$21)</f>
@@ -4738,7 +4827,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="B8" s="5" t="str">
         <f aca="false">COUNTIF('Pruebas Alfa'!$G$4:$G$20,"Aprobada")&amp;" de "&amp;COUNTA('Pruebas Alfa'!$A$4:$A$20)</f>
@@ -4747,42 +4836,42 @@
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>470</v>
+        <v>479</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>471</v>
+        <v>480</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>472</v>
+        <v>481</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>473</v>
+        <v>482</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>474</v>
+        <v>483</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>475</v>
+        <v>484</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>476</v>
+        <v>485</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>477</v>
+        <v>486</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>478</v>
+        <v>487</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>479</v>
+        <v>488</v>
       </c>
     </row>
   </sheetData>
@@ -4823,7 +4912,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>480</v>
+        <v>489</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4841,7 +4930,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>481</v>
+        <v>490</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4859,43 +4948,43 @@
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>482</v>
+        <v>491</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>483</v>
+        <v>492</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>484</v>
+        <v>493</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>485</v>
+        <v>494</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>486</v>
+        <v>495</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>487</v>
+        <v>496</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>488</v>
+        <v>497</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>490</v>
+        <v>499</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>491</v>
+        <v>500</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>492</v>
+        <v>501</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>4</v>
@@ -4903,7 +4992,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>493</v>
+        <v>502</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="5"/>
@@ -4921,7 +5010,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>494</v>
+        <v>503</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="5"/>
@@ -4939,7 +5028,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>495</v>
+        <v>504</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="5"/>
@@ -4957,7 +5046,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>496</v>
+        <v>505</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="5"/>
@@ -4975,7 +5064,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>497</v>
+        <v>506</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="5"/>
@@ -4993,7 +5082,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>498</v>
+        <v>507</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="5"/>
@@ -5011,7 +5100,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="5"/>
@@ -5029,7 +5118,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="5"/>
@@ -5047,7 +5136,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>501</v>
+        <v>510</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="5"/>
@@ -5065,7 +5154,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="5"/>
@@ -5083,7 +5172,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>503</v>
+        <v>512</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="5"/>
@@ -5101,7 +5190,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="5"/>
@@ -5119,7 +5208,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>505</v>
+        <v>514</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="5"/>
@@ -5137,7 +5226,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>506</v>
+        <v>515</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="5"/>
@@ -5155,7 +5244,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>507</v>
+        <v>516</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="5"/>
@@ -5173,7 +5262,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F20" s="8" t="s">
-        <v>508</v>
+        <v>517</v>
       </c>
       <c r="H20" s="19" t="n">
         <f aca="false">COUNTA(C4:C18)</f>
@@ -5182,7 +5271,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F21" s="8" t="s">
-        <v>509</v>
+        <v>518</v>
       </c>
       <c r="H21" s="0" t="str">
         <f aca="false">IF(COUNT(H4:H18)=0,"",ROUND(AVERAGE(H4:H18),1))</f>
@@ -5191,7 +5280,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F22" s="8" t="s">
-        <v>510</v>
+        <v>519</v>
       </c>
       <c r="H22" s="0" t="str">
         <f aca="false">IF(COUNT(I4:I18)=0,"",ROUND(AVERAGE(I4:I18),1))</f>
@@ -5200,7 +5289,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F23" s="8" t="s">
-        <v>511</v>
+        <v>520</v>
       </c>
       <c r="H23" s="0" t="str">
         <f aca="false">IF(COUNT(J4:J18)=0,"",ROUND(AVERAGE(J4:J18),1))</f>
@@ -5209,7 +5298,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F24" s="8" t="s">
-        <v>512</v>
+        <v>521</v>
       </c>
       <c r="H24" s="19" t="n">
         <f aca="false">COUNTIF(F4:F18,"Terminó el juego")</f>
@@ -5298,7 +5387,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5309,7 +5398,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5323,22 +5412,22 @@
         <v>6</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>4</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5359,10 +5448,10 @@
         <v>9</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5383,10 +5472,10 @@
         <v>35</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5407,10 +5496,10 @@
         <v>62</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5431,10 +5520,10 @@
         <v>62</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -5483,7 +5572,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -5498,7 +5587,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5511,7 +5600,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5524,48 +5613,48 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>15</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>9</v>
@@ -5582,19 +5671,19 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>92</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>90</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>9</v>
@@ -5611,19 +5700,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>9</v>
@@ -5640,19 +5729,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>9</v>
@@ -5669,19 +5758,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>9</v>
@@ -5698,19 +5787,19 @@
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>9</v>
@@ -5727,19 +5816,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>15</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>9</v>
@@ -5756,19 +5845,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>14</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>9</v>
@@ -5785,19 +5874,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>9</v>
@@ -5814,19 +5903,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>8</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>9</v>
@@ -5843,19 +5932,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B14" s="4" t="n">
         <v>10</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>9</v>
@@ -5872,19 +5961,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>11</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>9</v>
@@ -5901,19 +5990,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>12</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>9</v>
@@ -5930,19 +6019,19 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>15</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>9</v>
@@ -5959,19 +6048,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B18" s="4" t="n">
         <v>18</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>9</v>
@@ -5988,19 +6077,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B19" s="4" t="n">
         <v>20</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>9</v>
@@ -6017,19 +6106,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B20" s="4" t="n">
         <v>19</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>9</v>
@@ -6046,19 +6135,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B21" s="4" t="n">
         <v>19</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>9</v>
@@ -6075,19 +6164,19 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B22" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>9</v>
@@ -6104,19 +6193,19 @@
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B23" s="4" t="n">
         <v>23</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>9</v>
@@ -6133,19 +6222,19 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B24" s="4" t="n">
         <v>13</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>9</v>
@@ -6162,19 +6251,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B25" s="4" t="n">
         <v>11</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>9</v>
@@ -6191,19 +6280,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B26" s="4" t="n">
         <v>9</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>9</v>
@@ -6220,19 +6309,19 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B27" s="4" t="n">
         <v>22</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>9</v>
@@ -6249,19 +6338,19 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B28" s="4" t="n">
         <v>16</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F28" s="4" t="s">
         <v>9</v>
@@ -6278,19 +6367,19 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B29" s="4" t="n">
         <v>17</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>9</v>
@@ -6307,19 +6396,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B30" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F30" s="4" t="s">
         <v>9</v>
@@ -6336,19 +6425,19 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B31" s="4" t="n">
         <v>18</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>9</v>
@@ -6365,19 +6454,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B32" s="4" t="n">
         <v>11</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>9</v>
@@ -6394,19 +6483,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B33" s="4" t="n">
         <v>24</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F33" s="4" t="s">
         <v>9</v>
@@ -6423,19 +6512,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B34" s="4" t="n">
         <v>25</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>9</v>
@@ -6452,19 +6541,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B35" s="4" t="n">
         <v>14</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F35" s="4" t="s">
         <v>35</v>
@@ -6479,19 +6568,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B36" s="4" t="n">
         <v>24</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>35</v>
@@ -6506,19 +6595,19 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B37" s="4" t="n">
         <v>25</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>9</v>
@@ -6535,19 +6624,19 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B38" s="4" t="n">
         <v>14</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>62</v>
@@ -6560,19 +6649,19 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B39" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>9</v>
@@ -6589,19 +6678,19 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B40" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>9</v>
@@ -6618,19 +6707,19 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B41" s="4" t="n">
         <v>20</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F41" s="4" t="s">
         <v>9</v>
@@ -6647,19 +6736,19 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B42" s="4" t="n">
         <v>25</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>9</v>
@@ -6676,19 +6765,19 @@
     </row>
     <row r="43" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B43" s="4" t="n">
         <v>27</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>9</v>
@@ -6705,19 +6794,19 @@
     </row>
     <row r="44" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B44" s="4" t="n">
         <v>10</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F44" s="4" t="s">
         <v>9</v>
@@ -6734,19 +6823,19 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B45" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F45" s="4" t="s">
         <v>9</v>
@@ -6763,19 +6852,19 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B46" s="4" t="n">
         <v>23</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F46" s="4" t="s">
         <v>9</v>
@@ -6792,19 +6881,19 @@
     </row>
     <row r="47" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B47" s="4" t="n">
         <v>19</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F47" s="4" t="s">
         <v>9</v>
@@ -6821,19 +6910,19 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B48" s="4" t="n">
         <v>27</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F48" s="4" t="s">
         <v>9</v>
@@ -6850,19 +6939,19 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B49" s="4" t="n">
         <v>24</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F49" s="4" t="s">
         <v>9</v>
@@ -6879,19 +6968,19 @@
     </row>
     <row r="50" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B50" s="4" t="n">
         <v>14</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F50" s="4" t="s">
         <v>9</v>
@@ -6908,19 +6997,19 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B51" s="4" t="n">
         <v>25</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F51" s="4" t="s">
         <v>9</v>
@@ -6935,31 +7024,60 @@
         <v>46316</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F53" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="G53" s="8" t="n">
-        <f aca="false">SUM(G4:G51)</f>
-        <v>192</v>
+    <row r="52" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B52" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G52" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H52" s="6" t="n">
+        <v>46317</v>
+      </c>
+      <c r="I52" s="6" t="n">
+        <v>46317</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F54" s="8" t="s">
-        <v>186</v>
-      </c>
-      <c r="G54" s="8" t="str">
-        <f aca="false">COUNTIF(F4:F51,"Terminado")&amp;" de "&amp;COUNTA(A4:A51)</f>
-        <v>45 de 48</v>
+        <v>189</v>
+      </c>
+      <c r="G54" s="8" t="n">
+        <f aca="false">SUM(G4:G52)</f>
+        <v>198</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F55" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="G55" s="9" t="n">
-        <f aca="false">SUMIF(F4:F51,"Terminado",G4:G51)/G53</f>
-        <v>0.953125</v>
+        <v>190</v>
+      </c>
+      <c r="G55" s="8" t="str">
+        <f aca="false">COUNTIF(F4:F52,"Terminado")&amp;" de "&amp;COUNTA(A4:A52)</f>
+        <v>46 de 49</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F56" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="G56" s="9" t="n">
+        <f aca="false">SUMIF(F4:F52,"Terminado",G4:G52)/G54</f>
+        <v>0.954545454545455</v>
       </c>
     </row>
   </sheetData>
@@ -6967,7 +7085,7 @@
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F4:F51">
+  <conditionalFormatting sqref="F4:F52">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"Terminado"</formula>
     </cfRule>
@@ -6994,7 +7112,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F4:F51" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F4:F52" type="list">
       <formula1>"Terminado,En desarrollo,Planeado"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -7014,7 +7132,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -7023,7 +7141,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7031,7 +7149,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7039,16 +7157,16 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7056,13 +7174,13 @@
         <v>46284</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7070,13 +7188,13 @@
         <v>46295</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7084,13 +7202,13 @@
         <v>46299</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7098,13 +7216,13 @@
         <v>46300</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7112,13 +7230,13 @@
         <v>46302</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7126,13 +7244,13 @@
         <v>46308</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7140,13 +7258,13 @@
         <v>46310</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7154,13 +7272,13 @@
         <v>46315</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7168,13 +7286,27 @@
         <v>46316</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>220</v>
+        <v>224</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -7207,14 +7339,14 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7222,10 +7354,10 @@
         <v>4</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7233,12 +7365,12 @@
         <v>9</v>
       </c>
       <c r="B4" s="13" t="n">
-        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$30,A4)</f>
-        <v>24</v>
+        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$31,A4)</f>
+        <v>25</v>
       </c>
       <c r="C4" s="14" t="n">
         <f aca="false">IF(SUM($B$4:$B$7)=0,0,B4/SUM($B$4:$B$7))</f>
-        <v>0.888888888888889</v>
+        <v>0.892857142857143</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7246,12 +7378,12 @@
         <v>35</v>
       </c>
       <c r="B5" s="13" t="n">
-        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$30,A5)</f>
+        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$31,A5)</f>
         <v>2</v>
       </c>
       <c r="C5" s="14" t="n">
         <f aca="false">IF(SUM($B$4:$B$7)=0,0,B5/SUM($B$4:$B$7))</f>
-        <v>0.0740740740740741</v>
+        <v>0.0714285714285714</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7259,20 +7391,20 @@
         <v>62</v>
       </c>
       <c r="B6" s="13" t="n">
-        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$30,A6)</f>
+        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$31,A6)</f>
         <v>1</v>
       </c>
       <c r="C6" s="14" t="n">
         <f aca="false">IF(SUM($B$4:$B$7)=0,0,B6/SUM($B$4:$B$7))</f>
-        <v>0.037037037037037</v>
+        <v>0.0357142857142857</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="B7" s="13" t="n">
-        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$30,A7)</f>
+        <f aca="false">COUNTIF('Feature Log'!$C$4:$C$31,A7)</f>
         <v>0</v>
       </c>
       <c r="C7" s="14" t="n">
@@ -7282,11 +7414,11 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="B8" s="15" t="n">
         <f aca="false">SUM(B4:B7)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -7309,7 +7441,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -7320,7 +7452,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7328,7 +7460,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7338,16 +7470,16 @@
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7355,16 +7487,16 @@
         <v>46284</v>
       </c>
       <c r="B4" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A4)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>192</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$54*('Sprint Plan'!$D$5-A4)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>198</v>
       </c>
       <c r="C4" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A4)</f>
-        <v>192</v>
+        <f aca="false">'Sprint Backlog'!$G$54-SUMIFS('Sprint Backlog'!$G$4:$G$52,'Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A4)</f>
+        <v>198</v>
       </c>
       <c r="D4" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A4)</f>
-        <v>48</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-COUNTIFS('Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A4)</f>
+        <v>49</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7372,16 +7504,16 @@
         <v>46288</v>
       </c>
       <c r="B5" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A5)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>173.3</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$54*('Sprint Plan'!$D$5-A5)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>178.7</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A5)</f>
-        <v>192</v>
+        <f aca="false">'Sprint Backlog'!$G$54-SUMIFS('Sprint Backlog'!$G$4:$G$52,'Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A5)</f>
+        <v>198</v>
       </c>
       <c r="D5" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A5)</f>
-        <v>48</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-COUNTIFS('Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A5)</f>
+        <v>49</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7389,16 +7521,16 @@
         <v>46291</v>
       </c>
       <c r="B6" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A6)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>159.2</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$54*('Sprint Plan'!$D$5-A6)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>164.2</v>
       </c>
       <c r="C6" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A6)</f>
-        <v>192</v>
+        <f aca="false">'Sprint Backlog'!$G$54-SUMIFS('Sprint Backlog'!$G$4:$G$52,'Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A6)</f>
+        <v>198</v>
       </c>
       <c r="D6" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A6)</f>
-        <v>48</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-COUNTIFS('Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A6)</f>
+        <v>49</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7406,16 +7538,16 @@
         <v>46295</v>
       </c>
       <c r="B7" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A7)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>140.5</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$54*('Sprint Plan'!$D$5-A7)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>144.9</v>
       </c>
       <c r="C7" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A7)</f>
-        <v>154</v>
+        <f aca="false">'Sprint Backlog'!$G$54-SUMIFS('Sprint Backlog'!$G$4:$G$52,'Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A7)</f>
+        <v>160</v>
       </c>
       <c r="D7" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A7)</f>
-        <v>41</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-COUNTIFS('Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A7)</f>
+        <v>42</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7423,16 +7555,16 @@
         <v>46299</v>
       </c>
       <c r="B8" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A8)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>121.8</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$54*('Sprint Plan'!$D$5-A8)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>125.6</v>
       </c>
       <c r="C8" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A8)</f>
-        <v>101</v>
+        <f aca="false">'Sprint Backlog'!$G$54-SUMIFS('Sprint Backlog'!$G$4:$G$52,'Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A8)</f>
+        <v>107</v>
       </c>
       <c r="D8" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A8)</f>
-        <v>32</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-COUNTIFS('Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A8)</f>
+        <v>33</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7440,16 +7572,16 @@
         <v>46300</v>
       </c>
       <c r="B9" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A9)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>117.1</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$54*('Sprint Plan'!$D$5-A9)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>120.7</v>
       </c>
       <c r="C9" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A9)</f>
-        <v>51</v>
+        <f aca="false">'Sprint Backlog'!$G$54-SUMIFS('Sprint Backlog'!$G$4:$G$52,'Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A9)</f>
+        <v>57</v>
       </c>
       <c r="D9" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A9)</f>
-        <v>20</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-COUNTIFS('Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A9)</f>
+        <v>21</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7457,16 +7589,16 @@
         <v>46302</v>
       </c>
       <c r="B10" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A10)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>107.7</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$54*('Sprint Plan'!$D$5-A10)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>111.1</v>
       </c>
       <c r="C10" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A10)</f>
-        <v>42</v>
+        <f aca="false">'Sprint Backlog'!$G$54-SUMIFS('Sprint Backlog'!$G$4:$G$52,'Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A10)</f>
+        <v>48</v>
       </c>
       <c r="D10" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A10)</f>
-        <v>16</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-COUNTIFS('Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A10)</f>
+        <v>17</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7474,16 +7606,16 @@
         <v>46308</v>
       </c>
       <c r="B11" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A11)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>79.6</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$54*('Sprint Plan'!$D$5-A11)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>82.1</v>
       </c>
       <c r="C11" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A11)</f>
-        <v>29</v>
+        <f aca="false">'Sprint Backlog'!$G$54-SUMIFS('Sprint Backlog'!$G$4:$G$52,'Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A11)</f>
+        <v>35</v>
       </c>
       <c r="D11" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A11)</f>
-        <v>12</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-COUNTIFS('Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A11)</f>
+        <v>13</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7491,16 +7623,16 @@
         <v>46310</v>
       </c>
       <c r="B12" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A12)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>70.2</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$54*('Sprint Plan'!$D$5-A12)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>72.4</v>
       </c>
       <c r="C12" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A12)</f>
-        <v>18</v>
+        <f aca="false">'Sprint Backlog'!$G$54-SUMIFS('Sprint Backlog'!$G$4:$G$52,'Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A12)</f>
+        <v>24</v>
       </c>
       <c r="D12" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A12)</f>
-        <v>7</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-COUNTIFS('Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A12)</f>
+        <v>8</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7508,39 +7640,56 @@
         <v>46316</v>
       </c>
       <c r="B13" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A13)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>42.1</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$54*('Sprint Plan'!$D$5-A13)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>43.5</v>
       </c>
       <c r="C13" s="13" t="n">
-        <f aca="false">'Sprint Backlog'!$G$53-SUMIFS('Sprint Backlog'!$G$4:$G$51,'Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A13)</f>
-        <v>9</v>
+        <f aca="false">'Sprint Backlog'!$G$54-SUMIFS('Sprint Backlog'!$G$4:$G$52,'Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A13)</f>
+        <v>15</v>
       </c>
       <c r="D13" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-COUNTIFS('Sprint Backlog'!$F$4:$F$51,"Terminado",'Sprint Backlog'!$I$4:$I$51,"&lt;="&amp;A13)</f>
-        <v>3</v>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-COUNTIFS('Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A13)</f>
+        <v>4</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="n">
-        <v>46320</v>
+        <v>46317</v>
       </c>
       <c r="B14" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A14)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>23.4</v>
-      </c>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
+        <f aca="false">ROUND('Sprint Backlog'!$G$54*('Sprint Plan'!$D$5-A14)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>38.6</v>
+      </c>
+      <c r="C14" s="13" t="n">
+        <f aca="false">'Sprint Backlog'!$G$54-SUMIFS('Sprint Backlog'!$G$4:$G$52,'Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A14)</f>
+        <v>9</v>
+      </c>
+      <c r="D14" s="13" t="n">
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-COUNTIFS('Sprint Backlog'!$F$4:$F$52,"Terminado",'Sprint Backlog'!$I$4:$I$52,"&lt;="&amp;A14)</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="n">
-        <v>46325</v>
+        <v>46320</v>
       </c>
       <c r="B15" s="13" t="n">
-        <f aca="false">ROUND('Sprint Backlog'!$G$53*('Sprint Plan'!$D$5-A15)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
-        <v>0</v>
+        <f aca="false">ROUND('Sprint Backlog'!$G$54*('Sprint Plan'!$D$5-A15)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>24.1</v>
       </c>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="17" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B16" s="13" t="n">
+        <f aca="false">ROUND('Sprint Backlog'!$G$54*('Sprint Plan'!$D$5-A16)/('Sprint Plan'!$D$5-'Sprint Plan'!$B$5),1)</f>
+        <v>0</v>
+      </c>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -7563,7 +7712,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -7573,25 +7722,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7601,10 +7750,10 @@
       </c>
       <c r="B4" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D4</f>
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C4" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B4</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-B4</f>
         <v>0</v>
       </c>
     </row>
@@ -7615,10 +7764,10 @@
       </c>
       <c r="B5" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D5</f>
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C5" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B5</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-B5</f>
         <v>0</v>
       </c>
     </row>
@@ -7629,10 +7778,10 @@
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D6</f>
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C6" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B6</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-B6</f>
         <v>0</v>
       </c>
     </row>
@@ -7643,10 +7792,10 @@
       </c>
       <c r="B7" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D7</f>
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C7" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B7</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-B7</f>
         <v>7</v>
       </c>
     </row>
@@ -7657,10 +7806,10 @@
       </c>
       <c r="B8" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D8</f>
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C8" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B8</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-B8</f>
         <v>16</v>
       </c>
     </row>
@@ -7671,10 +7820,10 @@
       </c>
       <c r="B9" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D9</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B9</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-B9</f>
         <v>28</v>
       </c>
     </row>
@@ -7685,10 +7834,10 @@
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D10</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C10" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B10</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-B10</f>
         <v>32</v>
       </c>
     </row>
@@ -7699,10 +7848,10 @@
       </c>
       <c r="B11" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D11</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C11" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B11</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-B11</f>
         <v>36</v>
       </c>
     </row>
@@ -7713,10 +7862,10 @@
       </c>
       <c r="B12" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D12</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C12" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B12</f>
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-B12</f>
         <v>41</v>
       </c>
     </row>
@@ -7727,11 +7876,25 @@
       </c>
       <c r="B13" s="13" t="n">
         <f aca="false">'Burn-down Chart'!D13</f>
+        <v>4</v>
+      </c>
+      <c r="C13" s="13" t="n">
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-B13</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="17" t="n">
+        <f aca="false">'Burn-down Chart'!A14</f>
+        <v>46317</v>
+      </c>
+      <c r="B14" s="13" t="n">
+        <f aca="false">'Burn-down Chart'!D14</f>
         <v>3</v>
       </c>
-      <c r="C13" s="13" t="n">
-        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$51)-B13</f>
-        <v>45</v>
+      <c r="C14" s="13" t="n">
+        <f aca="false">COUNTA('Sprint Backlog'!$A$4:$A$52)-B14</f>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -7769,7 +7932,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -7781,7 +7944,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7793,16 +7956,16 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>4</v>
@@ -7811,27 +7974,27 @@
         <v>2</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>15</v>
@@ -7840,24 +8003,24 @@
         <v>46299</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>14</v>
@@ -7866,24 +8029,24 @@
         <v>46300</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>253</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>246</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>19</v>
@@ -7892,24 +8055,24 @@
         <v>46300</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>15</v>
@@ -7918,24 +8081,24 @@
         <v>46300</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>17</v>
@@ -7944,24 +8107,24 @@
         <v>46300</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>11</v>
@@ -7970,24 +8133,24 @@
         <v>46300</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>18</v>
@@ -7996,24 +8159,24 @@
         <v>46300</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>13</v>
@@ -8022,24 +8185,24 @@
         <v>46300</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>19</v>
@@ -8048,24 +8211,24 @@
         <v>46300</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F13" s="4" t="n">
         <v>22</v>
@@ -8074,24 +8237,24 @@
         <v>46300</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>17</v>
@@ -8100,24 +8263,24 @@
         <v>46300</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>11</v>
@@ -8126,24 +8289,24 @@
         <v>46302</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F16" s="4" t="n">
         <v>20</v>
@@ -8152,24 +8315,24 @@
         <v>46302</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="F17" s="4" t="n">
         <v>21</v>
@@ -8178,24 +8341,24 @@
         <v>46302</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F18" s="4" t="n">
         <v>1</v>
@@ -8204,24 +8367,24 @@
         <v>46308</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F19" s="4" t="n">
         <v>10</v>
@@ -8230,24 +8393,24 @@
         <v>46310</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F20" s="4" t="n">
         <v>1</v>
@@ -8256,24 +8419,24 @@
         <v>46310</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F21" s="4" t="n">
         <v>23</v>
@@ -8282,12 +8445,12 @@
         <v>46310</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D23" s="8" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="E23" s="8" t="str">
         <f aca="false">COUNTIF(E4:E21,"Corregido")&amp;" de "&amp;COUNTA(A4:A21)</f>
@@ -8354,7 +8517,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8365,7 +8528,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -8376,22 +8539,22 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>4</v>
@@ -8399,388 +8562,388 @@
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>322</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>323</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>324</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>320</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>20</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="D7" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>327</v>
       </c>
-      <c r="E7" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>320</v>
-      </c>
       <c r="G7" s="4" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>19</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>17</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>13</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>16</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="F12" s="5"/>
       <c r="G12" s="4" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="4" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="B14" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="D14" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>360</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>361</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>362</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>11</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>366</v>
+        <v>373</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>367</v>
+        <v>374</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>23</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>370</v>
+        <v>377</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>371</v>
+        <v>378</v>
       </c>
       <c r="F16" s="5"/>
       <c r="G16" s="4" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>24</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>376</v>
+        <v>383</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="B18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="B19" s="4" t="n">
         <v>27</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="F19" s="5"/>
       <c r="G19" s="4" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="B20" s="4" t="n">
         <v>27</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="F20" s="5"/>
       <c r="G20" s="4" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F22" s="8" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="G22" s="8" t="str">
         <f aca="false">COUNTIF(G4:G20,"Aprobada")&amp;" de "&amp;COUNTA(A4:A20)</f>

</xml_diff>